<commit_message>
cai tien input: auto-detect sheet + tu sinh advisor profile, fix bugs
</commit_message>
<xml_diff>
--- a/Thong_tin_truong_Han_ky_thang_3_2027.xlsx
+++ b/Thong_tin_truong_Han_ky_thang_3_2027.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\phant\Desktop\Thư mục mới\thong-tin-truong-han\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2BB5E973-7475-4695-9939-5F2938E1CD0D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{122B0202-9B72-4C44-BF17-3774D4D2A7CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="884" firstSheet="11" activeTab="18" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,20 @@
     <sheet name="ĐH Jeonju" sheetId="20" r:id="rId19"/>
     <sheet name="Check list HS xin Visa D2-6" sheetId="19" r:id="rId20"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -2561,29 +2574,10 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="12" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="2" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="2"/>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="2" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="21" fillId="4" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -2591,12 +2585,6 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="6" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="4" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="7" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
@@ -2610,6 +2598,31 @@
     </xf>
     <xf numFmtId="0" fontId="23" fillId="8" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="4" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="2" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="6" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -2979,13 +2992,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="37.950000000000003" customHeight="1">
-      <c r="A1" s="51" t="s">
+      <c r="A1" s="60" t="s">
         <v>89</v>
       </c>
-      <c r="B1" s="48"/>
-      <c r="C1" s="48"/>
-      <c r="D1" s="48"/>
-      <c r="E1" s="48"/>
+      <c r="B1" s="61"/>
+      <c r="C1" s="61"/>
+      <c r="D1" s="61"/>
+      <c r="E1" s="61"/>
     </row>
     <row r="2" spans="1:5" ht="22.05" customHeight="1">
       <c r="A2" s="27" t="s">
@@ -3277,11 +3290,11 @@
       </c>
     </row>
     <row r="19" spans="1:5" ht="30" customHeight="1">
-      <c r="A19" s="48"/>
-      <c r="B19" s="48"/>
-      <c r="C19" s="48"/>
-      <c r="D19" s="48"/>
-      <c r="E19" s="48"/>
+      <c r="A19" s="61"/>
+      <c r="B19" s="61"/>
+      <c r="C19" s="61"/>
+      <c r="D19" s="61"/>
+      <c r="E19" s="61"/>
     </row>
     <row r="20" spans="1:5" ht="22.05" customHeight="1">
       <c r="A20" s="45" t="s">
@@ -3548,20 +3561,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="30" customHeight="1">
-      <c r="A1" s="49" t="s">
+      <c r="A1" s="62" t="s">
         <v>258</v>
       </c>
-      <c r="B1" s="48"/>
+      <c r="B1" s="61"/>
     </row>
     <row r="2" spans="1:2" ht="6" customHeight="1">
-      <c r="A2" s="48"/>
-      <c r="B2" s="48"/>
+      <c r="A2" s="61"/>
+      <c r="B2" s="61"/>
     </row>
     <row r="3" spans="1:2" ht="30" customHeight="1">
-      <c r="A3" s="50" t="s">
+      <c r="A3" s="63" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="48"/>
+      <c r="B3" s="61"/>
     </row>
     <row r="4" spans="1:2" ht="18" customHeight="1">
       <c r="A4" s="17" t="s">
@@ -3620,14 +3633,14 @@
       </c>
     </row>
     <row r="11" spans="1:2" ht="6" customHeight="1">
-      <c r="A11" s="48"/>
-      <c r="B11" s="48"/>
+      <c r="A11" s="61"/>
+      <c r="B11" s="61"/>
     </row>
     <row r="12" spans="1:2" ht="30" customHeight="1">
-      <c r="A12" s="50" t="s">
+      <c r="A12" s="63" t="s">
         <v>13</v>
       </c>
-      <c r="B12" s="48"/>
+      <c r="B12" s="61"/>
     </row>
     <row r="13" spans="1:2" ht="409.2" customHeight="1">
       <c r="A13" s="17" t="s">
@@ -3638,14 +3651,14 @@
       </c>
     </row>
     <row r="14" spans="1:2">
-      <c r="A14" s="48"/>
-      <c r="B14" s="48"/>
+      <c r="A14" s="61"/>
+      <c r="B14" s="61"/>
     </row>
     <row r="15" spans="1:2" ht="30" customHeight="1">
-      <c r="A15" s="50" t="s">
+      <c r="A15" s="63" t="s">
         <v>16</v>
       </c>
-      <c r="B15" s="48"/>
+      <c r="B15" s="61"/>
     </row>
     <row r="16" spans="1:2" ht="105" customHeight="1">
       <c r="A16" s="17" t="s">
@@ -3672,14 +3685,14 @@
       </c>
     </row>
     <row r="19" spans="1:2" ht="6" customHeight="1">
-      <c r="A19" s="48"/>
-      <c r="B19" s="48"/>
+      <c r="A19" s="61"/>
+      <c r="B19" s="61"/>
     </row>
     <row r="20" spans="1:2" ht="30" customHeight="1">
-      <c r="A20" s="50" t="s">
+      <c r="A20" s="63" t="s">
         <v>23</v>
       </c>
-      <c r="B20" s="48"/>
+      <c r="B20" s="61"/>
     </row>
     <row r="21" spans="1:2" ht="345" customHeight="1">
       <c r="A21" s="17" t="s">
@@ -3690,14 +3703,14 @@
       </c>
     </row>
     <row r="22" spans="1:2" ht="6" customHeight="1">
-      <c r="A22" s="48"/>
-      <c r="B22" s="48"/>
+      <c r="A22" s="61"/>
+      <c r="B22" s="61"/>
     </row>
     <row r="23" spans="1:2" ht="30" customHeight="1">
-      <c r="A23" s="50" t="s">
+      <c r="A23" s="63" t="s">
         <v>26</v>
       </c>
-      <c r="B23" s="48"/>
+      <c r="B23" s="61"/>
     </row>
     <row r="24" spans="1:2" ht="135" customHeight="1">
       <c r="A24" s="17" t="s">
@@ -3724,14 +3737,14 @@
       </c>
     </row>
     <row r="27" spans="1:2" ht="6" customHeight="1">
-      <c r="A27" s="48"/>
-      <c r="B27" s="48"/>
+      <c r="A27" s="61"/>
+      <c r="B27" s="61"/>
     </row>
     <row r="28" spans="1:2" ht="30" customHeight="1">
-      <c r="A28" s="50" t="s">
+      <c r="A28" s="63" t="s">
         <v>33</v>
       </c>
-      <c r="B28" s="48"/>
+      <c r="B28" s="61"/>
     </row>
     <row r="29" spans="1:2" ht="18" customHeight="1">
       <c r="A29" s="17" t="s">
@@ -3750,14 +3763,14 @@
       </c>
     </row>
     <row r="31" spans="1:2" ht="6" customHeight="1">
-      <c r="A31" s="48"/>
-      <c r="B31" s="48"/>
+      <c r="A31" s="61"/>
+      <c r="B31" s="61"/>
     </row>
     <row r="32" spans="1:2" ht="25.05" customHeight="1">
-      <c r="A32" s="47" t="s">
+      <c r="A32" s="64" t="s">
         <v>37</v>
       </c>
-      <c r="B32" s="48"/>
+      <c r="B32" s="61"/>
     </row>
     <row r="33" spans="1:3" ht="19.95" customHeight="1">
       <c r="A33" s="20" t="s">
@@ -3983,20 +3996,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="30" customHeight="1">
-      <c r="A1" s="49" t="s">
+      <c r="A1" s="62" t="s">
         <v>268</v>
       </c>
-      <c r="B1" s="48"/>
+      <c r="B1" s="61"/>
     </row>
     <row r="2" spans="1:2">
-      <c r="A2" s="48"/>
-      <c r="B2" s="48"/>
+      <c r="A2" s="61"/>
+      <c r="B2" s="61"/>
     </row>
     <row r="3" spans="1:2" ht="30" customHeight="1">
-      <c r="A3" s="50" t="s">
+      <c r="A3" s="63" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="48"/>
+      <c r="B3" s="61"/>
     </row>
     <row r="4" spans="1:2" ht="15" customHeight="1">
       <c r="A4" s="17" t="s">
@@ -4055,14 +4068,14 @@
       </c>
     </row>
     <row r="11" spans="1:2">
-      <c r="A11" s="48"/>
-      <c r="B11" s="48"/>
+      <c r="A11" s="61"/>
+      <c r="B11" s="61"/>
     </row>
     <row r="12" spans="1:2" ht="30" customHeight="1">
-      <c r="A12" s="50" t="s">
+      <c r="A12" s="63" t="s">
         <v>13</v>
       </c>
-      <c r="B12" s="48"/>
+      <c r="B12" s="61"/>
     </row>
     <row r="13" spans="1:2" ht="193.2" customHeight="1">
       <c r="A13" s="17" t="s">
@@ -4073,14 +4086,14 @@
       </c>
     </row>
     <row r="14" spans="1:2">
-      <c r="A14" s="48"/>
-      <c r="B14" s="48"/>
+      <c r="A14" s="61"/>
+      <c r="B14" s="61"/>
     </row>
     <row r="15" spans="1:2" ht="30" customHeight="1">
-      <c r="A15" s="50" t="s">
+      <c r="A15" s="63" t="s">
         <v>16</v>
       </c>
-      <c r="B15" s="48"/>
+      <c r="B15" s="61"/>
     </row>
     <row r="16" spans="1:2" ht="105" customHeight="1">
       <c r="A16" s="17" t="s">
@@ -4107,14 +4120,14 @@
       </c>
     </row>
     <row r="19" spans="1:2">
-      <c r="A19" s="48"/>
-      <c r="B19" s="48"/>
+      <c r="A19" s="61"/>
+      <c r="B19" s="61"/>
     </row>
     <row r="20" spans="1:2" ht="30" customHeight="1">
-      <c r="A20" s="50" t="s">
+      <c r="A20" s="63" t="s">
         <v>23</v>
       </c>
-      <c r="B20" s="48"/>
+      <c r="B20" s="61"/>
     </row>
     <row r="21" spans="1:2" ht="317.39999999999998" customHeight="1">
       <c r="A21" s="17" t="s">
@@ -4125,14 +4138,14 @@
       </c>
     </row>
     <row r="22" spans="1:2">
-      <c r="A22" s="48"/>
-      <c r="B22" s="48"/>
+      <c r="A22" s="61"/>
+      <c r="B22" s="61"/>
     </row>
     <row r="23" spans="1:2" ht="30" customHeight="1">
-      <c r="A23" s="50" t="s">
+      <c r="A23" s="63" t="s">
         <v>26</v>
       </c>
-      <c r="B23" s="48"/>
+      <c r="B23" s="61"/>
     </row>
     <row r="24" spans="1:2" ht="105" customHeight="1">
       <c r="A24" s="17" t="s">
@@ -4159,14 +4172,14 @@
       </c>
     </row>
     <row r="27" spans="1:2">
-      <c r="A27" s="48"/>
-      <c r="B27" s="48"/>
+      <c r="A27" s="61"/>
+      <c r="B27" s="61"/>
     </row>
     <row r="28" spans="1:2" ht="30" customHeight="1">
-      <c r="A28" s="50" t="s">
+      <c r="A28" s="63" t="s">
         <v>33</v>
       </c>
-      <c r="B28" s="48"/>
+      <c r="B28" s="61"/>
     </row>
     <row r="29" spans="1:2" ht="15" customHeight="1">
       <c r="A29" s="17" t="s">
@@ -4185,14 +4198,14 @@
       </c>
     </row>
     <row r="31" spans="1:2">
-      <c r="A31" s="48"/>
-      <c r="B31" s="48"/>
+      <c r="A31" s="61"/>
+      <c r="B31" s="61"/>
     </row>
     <row r="32" spans="1:2" ht="25.05" customHeight="1">
-      <c r="A32" s="47" t="s">
+      <c r="A32" s="64" t="s">
         <v>37</v>
       </c>
-      <c r="B32" s="48"/>
+      <c r="B32" s="61"/>
     </row>
     <row r="33" spans="1:3" ht="19.95" customHeight="1">
       <c r="A33" s="20" t="s">
@@ -4419,20 +4432,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="30" customHeight="1">
-      <c r="A1" s="49" t="s">
+      <c r="A1" s="62" t="s">
         <v>281</v>
       </c>
-      <c r="B1" s="48"/>
+      <c r="B1" s="61"/>
     </row>
     <row r="2" spans="1:2">
-      <c r="A2" s="48"/>
-      <c r="B2" s="48"/>
+      <c r="A2" s="61"/>
+      <c r="B2" s="61"/>
     </row>
     <row r="3" spans="1:2" ht="30" customHeight="1">
-      <c r="A3" s="50" t="s">
+      <c r="A3" s="63" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="48"/>
+      <c r="B3" s="61"/>
     </row>
     <row r="4" spans="1:2" ht="15" customHeight="1">
       <c r="A4" s="17" t="s">
@@ -4491,14 +4504,14 @@
       </c>
     </row>
     <row r="11" spans="1:2">
-      <c r="A11" s="48"/>
-      <c r="B11" s="48"/>
+      <c r="A11" s="61"/>
+      <c r="B11" s="61"/>
     </row>
     <row r="12" spans="1:2" ht="30" customHeight="1">
-      <c r="A12" s="50" t="s">
+      <c r="A12" s="63" t="s">
         <v>13</v>
       </c>
-      <c r="B12" s="48"/>
+      <c r="B12" s="61"/>
     </row>
     <row r="13" spans="1:2" ht="150" customHeight="1">
       <c r="A13" s="17" t="s">
@@ -4509,14 +4522,14 @@
       </c>
     </row>
     <row r="14" spans="1:2">
-      <c r="A14" s="48"/>
-      <c r="B14" s="48"/>
+      <c r="A14" s="61"/>
+      <c r="B14" s="61"/>
     </row>
     <row r="15" spans="1:2" ht="30" customHeight="1">
-      <c r="A15" s="50" t="s">
+      <c r="A15" s="63" t="s">
         <v>16</v>
       </c>
-      <c r="B15" s="48"/>
+      <c r="B15" s="61"/>
     </row>
     <row r="16" spans="1:2" ht="105" customHeight="1">
       <c r="A16" s="17" t="s">
@@ -4543,14 +4556,14 @@
       </c>
     </row>
     <row r="19" spans="1:2">
-      <c r="A19" s="48"/>
-      <c r="B19" s="48"/>
+      <c r="A19" s="61"/>
+      <c r="B19" s="61"/>
     </row>
     <row r="20" spans="1:2" ht="30" customHeight="1">
-      <c r="A20" s="50" t="s">
+      <c r="A20" s="63" t="s">
         <v>23</v>
       </c>
-      <c r="B20" s="48"/>
+      <c r="B20" s="61"/>
     </row>
     <row r="21" spans="1:2" ht="317.39999999999998" customHeight="1">
       <c r="A21" s="17" t="s">
@@ -4561,14 +4574,14 @@
       </c>
     </row>
     <row r="22" spans="1:2">
-      <c r="A22" s="48"/>
-      <c r="B22" s="48"/>
+      <c r="A22" s="61"/>
+      <c r="B22" s="61"/>
     </row>
     <row r="23" spans="1:2" ht="30" customHeight="1">
-      <c r="A23" s="50" t="s">
+      <c r="A23" s="63" t="s">
         <v>26</v>
       </c>
-      <c r="B23" s="48"/>
+      <c r="B23" s="61"/>
     </row>
     <row r="24" spans="1:2" ht="120" customHeight="1">
       <c r="A24" s="17" t="s">
@@ -4595,14 +4608,14 @@
       </c>
     </row>
     <row r="27" spans="1:2">
-      <c r="A27" s="48"/>
-      <c r="B27" s="48"/>
+      <c r="A27" s="61"/>
+      <c r="B27" s="61"/>
     </row>
     <row r="28" spans="1:2" ht="30" customHeight="1">
-      <c r="A28" s="50" t="s">
+      <c r="A28" s="63" t="s">
         <v>33</v>
       </c>
-      <c r="B28" s="48"/>
+      <c r="B28" s="61"/>
     </row>
     <row r="29" spans="1:2" ht="15" customHeight="1">
       <c r="A29" s="17" t="s">
@@ -4621,14 +4634,14 @@
       </c>
     </row>
     <row r="31" spans="1:2">
-      <c r="A31" s="48"/>
-      <c r="B31" s="48"/>
+      <c r="A31" s="61"/>
+      <c r="B31" s="61"/>
     </row>
     <row r="32" spans="1:2" ht="25.05" customHeight="1">
-      <c r="A32" s="47" t="s">
+      <c r="A32" s="64" t="s">
         <v>37</v>
       </c>
-      <c r="B32" s="48"/>
+      <c r="B32" s="61"/>
     </row>
     <row r="33" spans="1:3" ht="19.95" customHeight="1">
       <c r="A33" s="20" t="s">
@@ -4855,20 +4868,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="30" customHeight="1">
-      <c r="A1" s="49" t="s">
+      <c r="A1" s="62" t="s">
         <v>292</v>
       </c>
-      <c r="B1" s="48"/>
+      <c r="B1" s="61"/>
     </row>
     <row r="2" spans="1:2">
-      <c r="A2" s="48"/>
-      <c r="B2" s="48"/>
+      <c r="A2" s="61"/>
+      <c r="B2" s="61"/>
     </row>
     <row r="3" spans="1:2" ht="30" customHeight="1">
-      <c r="A3" s="50" t="s">
+      <c r="A3" s="63" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="48"/>
+      <c r="B3" s="61"/>
     </row>
     <row r="4" spans="1:2" ht="15" customHeight="1">
       <c r="A4" s="17" t="s">
@@ -4927,14 +4940,14 @@
       </c>
     </row>
     <row r="11" spans="1:2">
-      <c r="A11" s="48"/>
-      <c r="B11" s="48"/>
+      <c r="A11" s="61"/>
+      <c r="B11" s="61"/>
     </row>
     <row r="12" spans="1:2" ht="30" customHeight="1">
-      <c r="A12" s="50" t="s">
+      <c r="A12" s="63" t="s">
         <v>13</v>
       </c>
-      <c r="B12" s="48"/>
+      <c r="B12" s="61"/>
     </row>
     <row r="13" spans="1:2" ht="150" customHeight="1">
       <c r="A13" s="17" t="s">
@@ -4945,14 +4958,14 @@
       </c>
     </row>
     <row r="14" spans="1:2">
-      <c r="A14" s="48"/>
-      <c r="B14" s="48"/>
+      <c r="A14" s="61"/>
+      <c r="B14" s="61"/>
     </row>
     <row r="15" spans="1:2" ht="30" customHeight="1">
-      <c r="A15" s="50" t="s">
+      <c r="A15" s="63" t="s">
         <v>16</v>
       </c>
-      <c r="B15" s="48"/>
+      <c r="B15" s="61"/>
     </row>
     <row r="16" spans="1:2" ht="105" customHeight="1">
       <c r="A16" s="17" t="s">
@@ -4979,14 +4992,14 @@
       </c>
     </row>
     <row r="19" spans="1:2">
-      <c r="A19" s="48"/>
-      <c r="B19" s="48"/>
+      <c r="A19" s="61"/>
+      <c r="B19" s="61"/>
     </row>
     <row r="20" spans="1:2" ht="30" customHeight="1">
-      <c r="A20" s="50" t="s">
+      <c r="A20" s="63" t="s">
         <v>23</v>
       </c>
-      <c r="B20" s="48"/>
+      <c r="B20" s="61"/>
     </row>
     <row r="21" spans="1:2" ht="317.39999999999998" customHeight="1">
       <c r="A21" s="17" t="s">
@@ -4997,14 +5010,14 @@
       </c>
     </row>
     <row r="22" spans="1:2">
-      <c r="A22" s="48"/>
-      <c r="B22" s="48"/>
+      <c r="A22" s="61"/>
+      <c r="B22" s="61"/>
     </row>
     <row r="23" spans="1:2" ht="30" customHeight="1">
-      <c r="A23" s="50" t="s">
+      <c r="A23" s="63" t="s">
         <v>26</v>
       </c>
-      <c r="B23" s="48"/>
+      <c r="B23" s="61"/>
     </row>
     <row r="24" spans="1:2" ht="105" customHeight="1">
       <c r="A24" s="17" t="s">
@@ -5031,14 +5044,14 @@
       </c>
     </row>
     <row r="27" spans="1:2">
-      <c r="A27" s="48"/>
-      <c r="B27" s="48"/>
+      <c r="A27" s="61"/>
+      <c r="B27" s="61"/>
     </row>
     <row r="28" spans="1:2" ht="30" customHeight="1">
-      <c r="A28" s="50" t="s">
+      <c r="A28" s="63" t="s">
         <v>33</v>
       </c>
-      <c r="B28" s="48"/>
+      <c r="B28" s="61"/>
     </row>
     <row r="29" spans="1:2" ht="15" customHeight="1">
       <c r="A29" s="17" t="s">
@@ -5057,14 +5070,14 @@
       </c>
     </row>
     <row r="31" spans="1:2">
-      <c r="A31" s="48"/>
-      <c r="B31" s="48"/>
+      <c r="A31" s="61"/>
+      <c r="B31" s="61"/>
     </row>
     <row r="32" spans="1:2" ht="25.05" customHeight="1">
-      <c r="A32" s="47" t="s">
+      <c r="A32" s="64" t="s">
         <v>37</v>
       </c>
-      <c r="B32" s="48"/>
+      <c r="B32" s="61"/>
     </row>
     <row r="33" spans="1:3" ht="19.95" customHeight="1">
       <c r="A33" s="20" t="s">
@@ -5290,20 +5303,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="30" customHeight="1">
-      <c r="A1" s="49" t="s">
+      <c r="A1" s="62" t="s">
         <v>302</v>
       </c>
-      <c r="B1" s="48"/>
+      <c r="B1" s="61"/>
     </row>
     <row r="2" spans="1:2">
-      <c r="A2" s="48"/>
-      <c r="B2" s="48"/>
+      <c r="A2" s="61"/>
+      <c r="B2" s="61"/>
     </row>
     <row r="3" spans="1:2" ht="30" customHeight="1">
-      <c r="A3" s="50" t="s">
+      <c r="A3" s="63" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="48"/>
+      <c r="B3" s="61"/>
     </row>
     <row r="4" spans="1:2" ht="15" customHeight="1">
       <c r="A4" s="17" t="s">
@@ -5362,14 +5375,14 @@
       </c>
     </row>
     <row r="11" spans="1:2">
-      <c r="A11" s="48"/>
-      <c r="B11" s="48"/>
+      <c r="A11" s="61"/>
+      <c r="B11" s="61"/>
     </row>
     <row r="12" spans="1:2" ht="30" customHeight="1">
-      <c r="A12" s="50" t="s">
+      <c r="A12" s="63" t="s">
         <v>13</v>
       </c>
-      <c r="B12" s="48"/>
+      <c r="B12" s="61"/>
     </row>
     <row r="13" spans="1:2" ht="150" customHeight="1">
       <c r="A13" s="17" t="s">
@@ -5380,14 +5393,14 @@
       </c>
     </row>
     <row r="14" spans="1:2">
-      <c r="A14" s="48"/>
-      <c r="B14" s="48"/>
+      <c r="A14" s="61"/>
+      <c r="B14" s="61"/>
     </row>
     <row r="15" spans="1:2" ht="30" customHeight="1">
-      <c r="A15" s="50" t="s">
+      <c r="A15" s="63" t="s">
         <v>16</v>
       </c>
-      <c r="B15" s="48"/>
+      <c r="B15" s="61"/>
     </row>
     <row r="16" spans="1:2" ht="105" customHeight="1">
       <c r="A16" s="17" t="s">
@@ -5414,14 +5427,14 @@
       </c>
     </row>
     <row r="19" spans="1:2">
-      <c r="A19" s="48"/>
-      <c r="B19" s="48"/>
+      <c r="A19" s="61"/>
+      <c r="B19" s="61"/>
     </row>
     <row r="20" spans="1:2" ht="30" customHeight="1">
-      <c r="A20" s="50" t="s">
+      <c r="A20" s="63" t="s">
         <v>23</v>
       </c>
-      <c r="B20" s="48"/>
+      <c r="B20" s="61"/>
     </row>
     <row r="21" spans="1:2" ht="317.39999999999998" customHeight="1">
       <c r="A21" s="17" t="s">
@@ -5432,14 +5445,14 @@
       </c>
     </row>
     <row r="22" spans="1:2">
-      <c r="A22" s="48"/>
-      <c r="B22" s="48"/>
+      <c r="A22" s="61"/>
+      <c r="B22" s="61"/>
     </row>
     <row r="23" spans="1:2" ht="30" customHeight="1">
-      <c r="A23" s="50" t="s">
+      <c r="A23" s="63" t="s">
         <v>26</v>
       </c>
-      <c r="B23" s="48"/>
+      <c r="B23" s="61"/>
     </row>
     <row r="24" spans="1:2" ht="105" customHeight="1">
       <c r="A24" s="17" t="s">
@@ -5466,14 +5479,14 @@
       </c>
     </row>
     <row r="27" spans="1:2">
-      <c r="A27" s="48"/>
-      <c r="B27" s="48"/>
+      <c r="A27" s="61"/>
+      <c r="B27" s="61"/>
     </row>
     <row r="28" spans="1:2" ht="30" customHeight="1">
-      <c r="A28" s="50" t="s">
+      <c r="A28" s="63" t="s">
         <v>33</v>
       </c>
-      <c r="B28" s="48"/>
+      <c r="B28" s="61"/>
     </row>
     <row r="29" spans="1:2" ht="15" customHeight="1">
       <c r="A29" s="17" t="s">
@@ -5492,14 +5505,14 @@
       </c>
     </row>
     <row r="31" spans="1:2">
-      <c r="A31" s="48"/>
-      <c r="B31" s="48"/>
+      <c r="A31" s="61"/>
+      <c r="B31" s="61"/>
     </row>
     <row r="32" spans="1:2" ht="25.05" customHeight="1">
-      <c r="A32" s="47" t="s">
+      <c r="A32" s="64" t="s">
         <v>37</v>
       </c>
-      <c r="B32" s="48"/>
+      <c r="B32" s="61"/>
     </row>
     <row r="33" spans="1:3" ht="19.95" customHeight="1">
       <c r="A33" s="20" t="s">
@@ -5725,20 +5738,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="30" customHeight="1">
-      <c r="A1" s="49" t="s">
+      <c r="A1" s="62" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="48"/>
+      <c r="B1" s="61"/>
     </row>
     <row r="2" spans="1:2" ht="6" customHeight="1">
-      <c r="A2" s="48"/>
-      <c r="B2" s="48"/>
+      <c r="A2" s="61"/>
+      <c r="B2" s="61"/>
     </row>
     <row r="3" spans="1:2" ht="30" customHeight="1">
-      <c r="A3" s="50" t="s">
+      <c r="A3" s="63" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="48"/>
+      <c r="B3" s="61"/>
     </row>
     <row r="4" spans="1:2" ht="18" customHeight="1">
       <c r="A4" s="17" t="s">
@@ -5797,14 +5810,14 @@
       </c>
     </row>
     <row r="11" spans="1:2" ht="6" customHeight="1">
-      <c r="A11" s="48"/>
-      <c r="B11" s="48"/>
+      <c r="A11" s="61"/>
+      <c r="B11" s="61"/>
     </row>
     <row r="12" spans="1:2" ht="30" customHeight="1">
-      <c r="A12" s="50" t="s">
+      <c r="A12" s="63" t="s">
         <v>13</v>
       </c>
-      <c r="B12" s="48"/>
+      <c r="B12" s="61"/>
     </row>
     <row r="13" spans="1:2" ht="400.2" customHeight="1">
       <c r="A13" s="17" t="s">
@@ -5815,14 +5828,14 @@
       </c>
     </row>
     <row r="14" spans="1:2" ht="6" customHeight="1">
-      <c r="A14" s="48"/>
-      <c r="B14" s="48"/>
+      <c r="A14" s="61"/>
+      <c r="B14" s="61"/>
     </row>
     <row r="15" spans="1:2" ht="30" customHeight="1">
-      <c r="A15" s="50" t="s">
+      <c r="A15" s="63" t="s">
         <v>16</v>
       </c>
-      <c r="B15" s="48"/>
+      <c r="B15" s="61"/>
     </row>
     <row r="16" spans="1:2" ht="96.6" customHeight="1">
       <c r="A16" s="17" t="s">
@@ -5849,14 +5862,14 @@
       </c>
     </row>
     <row r="19" spans="1:2" ht="6" customHeight="1">
-      <c r="A19" s="48"/>
-      <c r="B19" s="48"/>
+      <c r="A19" s="61"/>
+      <c r="B19" s="61"/>
     </row>
     <row r="20" spans="1:2" ht="30" customHeight="1">
-      <c r="A20" s="50" t="s">
+      <c r="A20" s="63" t="s">
         <v>23</v>
       </c>
-      <c r="B20" s="48"/>
+      <c r="B20" s="61"/>
     </row>
     <row r="21" spans="1:2" ht="300" customHeight="1">
       <c r="A21" s="17" t="s">
@@ -5867,14 +5880,14 @@
       </c>
     </row>
     <row r="22" spans="1:2" ht="6" customHeight="1">
-      <c r="A22" s="48"/>
-      <c r="B22" s="48"/>
+      <c r="A22" s="61"/>
+      <c r="B22" s="61"/>
     </row>
     <row r="23" spans="1:2" ht="30" customHeight="1">
-      <c r="A23" s="50" t="s">
+      <c r="A23" s="63" t="s">
         <v>26</v>
       </c>
-      <c r="B23" s="48"/>
+      <c r="B23" s="61"/>
     </row>
     <row r="24" spans="1:2" ht="135" customHeight="1">
       <c r="A24" s="17" t="s">
@@ -5901,14 +5914,14 @@
       </c>
     </row>
     <row r="27" spans="1:2" ht="6" customHeight="1">
-      <c r="A27" s="48"/>
-      <c r="B27" s="48"/>
+      <c r="A27" s="61"/>
+      <c r="B27" s="61"/>
     </row>
     <row r="28" spans="1:2" ht="30" customHeight="1">
-      <c r="A28" s="50" t="s">
+      <c r="A28" s="63" t="s">
         <v>33</v>
       </c>
-      <c r="B28" s="48"/>
+      <c r="B28" s="61"/>
     </row>
     <row r="29" spans="1:2" ht="18" customHeight="1">
       <c r="A29" s="17" t="s">
@@ -5925,14 +5938,14 @@
       </c>
     </row>
     <row r="31" spans="1:2" ht="6" customHeight="1">
-      <c r="A31" s="48"/>
-      <c r="B31" s="48"/>
+      <c r="A31" s="61"/>
+      <c r="B31" s="61"/>
     </row>
     <row r="32" spans="1:2" ht="25.05" customHeight="1">
-      <c r="A32" s="47" t="s">
+      <c r="A32" s="64" t="s">
         <v>37</v>
       </c>
-      <c r="B32" s="48"/>
+      <c r="B32" s="61"/>
     </row>
     <row r="33" spans="1:3" ht="19.95" customHeight="1">
       <c r="A33" s="20" t="s">
@@ -6159,20 +6172,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="30" customHeight="1">
-      <c r="A1" s="49" t="s">
+      <c r="A1" s="62" t="s">
         <v>312</v>
       </c>
-      <c r="B1" s="48"/>
+      <c r="B1" s="61"/>
     </row>
     <row r="2" spans="1:2">
-      <c r="A2" s="48"/>
-      <c r="B2" s="48"/>
+      <c r="A2" s="61"/>
+      <c r="B2" s="61"/>
     </row>
     <row r="3" spans="1:2" ht="30" customHeight="1">
-      <c r="A3" s="50" t="s">
+      <c r="A3" s="63" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="48"/>
+      <c r="B3" s="61"/>
     </row>
     <row r="4" spans="1:2" ht="15" customHeight="1">
       <c r="A4" s="17" t="s">
@@ -6231,14 +6244,14 @@
       </c>
     </row>
     <row r="11" spans="1:2">
-      <c r="A11" s="48"/>
-      <c r="B11" s="48"/>
+      <c r="A11" s="61"/>
+      <c r="B11" s="61"/>
     </row>
     <row r="12" spans="1:2" ht="30" customHeight="1">
-      <c r="A12" s="50" t="s">
+      <c r="A12" s="63" t="s">
         <v>13</v>
       </c>
-      <c r="B12" s="48"/>
+      <c r="B12" s="61"/>
     </row>
     <row r="13" spans="1:2" ht="193.2" customHeight="1">
       <c r="A13" s="17" t="s">
@@ -6249,14 +6262,14 @@
       </c>
     </row>
     <row r="14" spans="1:2">
-      <c r="A14" s="48"/>
-      <c r="B14" s="48"/>
+      <c r="A14" s="61"/>
+      <c r="B14" s="61"/>
     </row>
     <row r="15" spans="1:2" ht="30" customHeight="1">
-      <c r="A15" s="50" t="s">
+      <c r="A15" s="63" t="s">
         <v>16</v>
       </c>
-      <c r="B15" s="48"/>
+      <c r="B15" s="61"/>
     </row>
     <row r="16" spans="1:2" ht="96.6" customHeight="1">
       <c r="A16" s="17" t="s">
@@ -6283,14 +6296,14 @@
       </c>
     </row>
     <row r="19" spans="1:2">
-      <c r="A19" s="48"/>
-      <c r="B19" s="48"/>
+      <c r="A19" s="61"/>
+      <c r="B19" s="61"/>
     </row>
     <row r="20" spans="1:2" ht="30" customHeight="1">
-      <c r="A20" s="50" t="s">
+      <c r="A20" s="63" t="s">
         <v>23</v>
       </c>
-      <c r="B20" s="48"/>
+      <c r="B20" s="61"/>
     </row>
     <row r="21" spans="1:2" ht="317.39999999999998" customHeight="1">
       <c r="A21" s="17" t="s">
@@ -6301,14 +6314,14 @@
       </c>
     </row>
     <row r="22" spans="1:2">
-      <c r="A22" s="48"/>
-      <c r="B22" s="48"/>
+      <c r="A22" s="61"/>
+      <c r="B22" s="61"/>
     </row>
     <row r="23" spans="1:2" ht="30" customHeight="1">
-      <c r="A23" s="50" t="s">
+      <c r="A23" s="63" t="s">
         <v>26</v>
       </c>
-      <c r="B23" s="48"/>
+      <c r="B23" s="61"/>
     </row>
     <row r="24" spans="1:2" ht="105" customHeight="1">
       <c r="A24" s="17" t="s">
@@ -6335,14 +6348,14 @@
       </c>
     </row>
     <row r="27" spans="1:2">
-      <c r="A27" s="48"/>
-      <c r="B27" s="48"/>
+      <c r="A27" s="61"/>
+      <c r="B27" s="61"/>
     </row>
     <row r="28" spans="1:2" ht="30" customHeight="1">
-      <c r="A28" s="50" t="s">
+      <c r="A28" s="63" t="s">
         <v>33</v>
       </c>
-      <c r="B28" s="48"/>
+      <c r="B28" s="61"/>
     </row>
     <row r="29" spans="1:2" ht="15" customHeight="1">
       <c r="A29" s="17" t="s">
@@ -6361,14 +6374,14 @@
       </c>
     </row>
     <row r="31" spans="1:2">
-      <c r="A31" s="48"/>
-      <c r="B31" s="48"/>
+      <c r="A31" s="61"/>
+      <c r="B31" s="61"/>
     </row>
     <row r="32" spans="1:2" ht="25.05" customHeight="1">
-      <c r="A32" s="47" t="s">
+      <c r="A32" s="64" t="s">
         <v>37</v>
       </c>
-      <c r="B32" s="48"/>
+      <c r="B32" s="61"/>
     </row>
     <row r="33" spans="1:3" ht="19.95" customHeight="1">
       <c r="A33" s="20" t="s">
@@ -6594,20 +6607,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="30" customHeight="1">
-      <c r="A1" s="49" t="s">
+      <c r="A1" s="62" t="s">
         <v>322</v>
       </c>
-      <c r="B1" s="48"/>
+      <c r="B1" s="61"/>
     </row>
     <row r="2" spans="1:2" ht="6" customHeight="1">
-      <c r="A2" s="48"/>
-      <c r="B2" s="48"/>
+      <c r="A2" s="61"/>
+      <c r="B2" s="61"/>
     </row>
     <row r="3" spans="1:2" ht="30" customHeight="1">
-      <c r="A3" s="50" t="s">
+      <c r="A3" s="63" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="48"/>
+      <c r="B3" s="61"/>
     </row>
     <row r="4" spans="1:2" ht="27.6" customHeight="1">
       <c r="A4" s="36" t="s">
@@ -6666,14 +6679,14 @@
       </c>
     </row>
     <row r="11" spans="1:2" ht="6" customHeight="1">
-      <c r="A11" s="48"/>
-      <c r="B11" s="48"/>
+      <c r="A11" s="61"/>
+      <c r="B11" s="61"/>
     </row>
     <row r="12" spans="1:2" ht="30" customHeight="1">
-      <c r="A12" s="50" t="s">
+      <c r="A12" s="63" t="s">
         <v>13</v>
       </c>
-      <c r="B12" s="48"/>
+      <c r="B12" s="61"/>
     </row>
     <row r="13" spans="1:2" ht="303.60000000000002" customHeight="1">
       <c r="A13" s="36" t="s">
@@ -6684,14 +6697,14 @@
       </c>
     </row>
     <row r="14" spans="1:2" ht="6" customHeight="1">
-      <c r="A14" s="48"/>
-      <c r="B14" s="48"/>
+      <c r="A14" s="61"/>
+      <c r="B14" s="61"/>
     </row>
     <row r="15" spans="1:2" ht="30" customHeight="1">
-      <c r="A15" s="50" t="s">
+      <c r="A15" s="63" t="s">
         <v>16</v>
       </c>
-      <c r="B15" s="48"/>
+      <c r="B15" s="61"/>
     </row>
     <row r="16" spans="1:2" ht="180" customHeight="1">
       <c r="A16" s="36" t="s">
@@ -6718,14 +6731,14 @@
       </c>
     </row>
     <row r="19" spans="1:2" ht="6" customHeight="1">
-      <c r="A19" s="48"/>
-      <c r="B19" s="48"/>
+      <c r="A19" s="61"/>
+      <c r="B19" s="61"/>
     </row>
     <row r="20" spans="1:2" ht="30" customHeight="1">
-      <c r="A20" s="50" t="s">
+      <c r="A20" s="63" t="s">
         <v>23</v>
       </c>
-      <c r="B20" s="48"/>
+      <c r="B20" s="61"/>
     </row>
     <row r="21" spans="1:2" ht="409.6" customHeight="1">
       <c r="A21" s="36" t="s">
@@ -6736,14 +6749,14 @@
       </c>
     </row>
     <row r="22" spans="1:2" ht="6" customHeight="1">
-      <c r="A22" s="48"/>
-      <c r="B22" s="48"/>
+      <c r="A22" s="61"/>
+      <c r="B22" s="61"/>
     </row>
     <row r="23" spans="1:2" ht="30" customHeight="1">
-      <c r="A23" s="50" t="s">
+      <c r="A23" s="63" t="s">
         <v>26</v>
       </c>
-      <c r="B23" s="48"/>
+      <c r="B23" s="61"/>
     </row>
     <row r="24" spans="1:2" ht="180" customHeight="1">
       <c r="A24" s="36" t="s">
@@ -6770,14 +6783,14 @@
       </c>
     </row>
     <row r="27" spans="1:2" ht="6" customHeight="1">
-      <c r="A27" s="48"/>
-      <c r="B27" s="48"/>
+      <c r="A27" s="61"/>
+      <c r="B27" s="61"/>
     </row>
     <row r="28" spans="1:2" ht="30" customHeight="1">
-      <c r="A28" s="50" t="s">
+      <c r="A28" s="63" t="s">
         <v>33</v>
       </c>
-      <c r="B28" s="48"/>
+      <c r="B28" s="61"/>
     </row>
     <row r="29" spans="1:2" ht="18" customHeight="1">
       <c r="A29" s="36" t="s">
@@ -6796,14 +6809,14 @@
       </c>
     </row>
     <row r="31" spans="1:2" ht="6" customHeight="1">
-      <c r="A31" s="48"/>
-      <c r="B31" s="48"/>
+      <c r="A31" s="61"/>
+      <c r="B31" s="61"/>
     </row>
     <row r="32" spans="1:2" ht="25.05" customHeight="1">
-      <c r="A32" s="47" t="s">
+      <c r="A32" s="64" t="s">
         <v>37</v>
       </c>
-      <c r="B32" s="48"/>
+      <c r="B32" s="61"/>
     </row>
     <row r="33" spans="1:3" ht="19.95" customHeight="1">
       <c r="A33" s="27" t="s">
@@ -7029,20 +7042,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="30" customHeight="1">
-      <c r="A1" s="49" t="s">
+      <c r="A1" s="62" t="s">
         <v>337</v>
       </c>
-      <c r="B1" s="48"/>
+      <c r="B1" s="61"/>
     </row>
     <row r="2" spans="1:2" ht="6" customHeight="1">
-      <c r="A2" s="48"/>
-      <c r="B2" s="48"/>
+      <c r="A2" s="61"/>
+      <c r="B2" s="61"/>
     </row>
     <row r="3" spans="1:2" ht="30" customHeight="1">
-      <c r="A3" s="50" t="s">
+      <c r="A3" s="63" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="48"/>
+      <c r="B3" s="61"/>
     </row>
     <row r="4" spans="1:2" ht="27.6" customHeight="1">
       <c r="A4" s="17" t="s">
@@ -7101,14 +7114,14 @@
       </c>
     </row>
     <row r="11" spans="1:2">
-      <c r="A11" s="48"/>
-      <c r="B11" s="48"/>
+      <c r="A11" s="61"/>
+      <c r="B11" s="61"/>
     </row>
     <row r="12" spans="1:2" ht="30" customHeight="1">
-      <c r="A12" s="50" t="s">
+      <c r="A12" s="63" t="s">
         <v>13</v>
       </c>
-      <c r="B12" s="48"/>
+      <c r="B12" s="61"/>
     </row>
     <row r="13" spans="1:2" ht="207" customHeight="1">
       <c r="A13" s="17" t="s">
@@ -7119,14 +7132,14 @@
       </c>
     </row>
     <row r="14" spans="1:2">
-      <c r="A14" s="48"/>
-      <c r="B14" s="48"/>
+      <c r="A14" s="61"/>
+      <c r="B14" s="61"/>
     </row>
     <row r="15" spans="1:2" ht="30" customHeight="1">
-      <c r="A15" s="50" t="s">
+      <c r="A15" s="63" t="s">
         <v>16</v>
       </c>
-      <c r="B15" s="48"/>
+      <c r="B15" s="61"/>
     </row>
     <row r="16" spans="1:2" ht="105" customHeight="1">
       <c r="A16" s="17" t="s">
@@ -7153,14 +7166,14 @@
       </c>
     </row>
     <row r="19" spans="1:2">
-      <c r="A19" s="48"/>
-      <c r="B19" s="48"/>
+      <c r="A19" s="61"/>
+      <c r="B19" s="61"/>
     </row>
     <row r="20" spans="1:2" ht="30" customHeight="1">
-      <c r="A20" s="50" t="s">
+      <c r="A20" s="63" t="s">
         <v>23</v>
       </c>
-      <c r="B20" s="48"/>
+      <c r="B20" s="61"/>
     </row>
     <row r="21" spans="1:2" ht="372.6" customHeight="1">
       <c r="A21" s="17" t="s">
@@ -7171,14 +7184,14 @@
       </c>
     </row>
     <row r="22" spans="1:2">
-      <c r="A22" s="48"/>
-      <c r="B22" s="48"/>
+      <c r="A22" s="61"/>
+      <c r="B22" s="61"/>
     </row>
     <row r="23" spans="1:2" ht="30" customHeight="1">
-      <c r="A23" s="50" t="s">
+      <c r="A23" s="63" t="s">
         <v>26</v>
       </c>
-      <c r="B23" s="48"/>
+      <c r="B23" s="61"/>
     </row>
     <row r="24" spans="1:2" ht="151.80000000000001" customHeight="1">
       <c r="A24" s="17" t="s">
@@ -7205,14 +7218,14 @@
       </c>
     </row>
     <row r="27" spans="1:2">
-      <c r="A27" s="48"/>
-      <c r="B27" s="48"/>
+      <c r="A27" s="61"/>
+      <c r="B27" s="61"/>
     </row>
     <row r="28" spans="1:2" ht="30" customHeight="1">
-      <c r="A28" s="50" t="s">
+      <c r="A28" s="63" t="s">
         <v>33</v>
       </c>
-      <c r="B28" s="48"/>
+      <c r="B28" s="61"/>
     </row>
     <row r="29" spans="1:2" ht="18" customHeight="1">
       <c r="A29" s="17" t="s">
@@ -7229,14 +7242,14 @@
       </c>
     </row>
     <row r="31" spans="1:2">
-      <c r="A31" s="48"/>
-      <c r="B31" s="48"/>
+      <c r="A31" s="61"/>
+      <c r="B31" s="61"/>
     </row>
     <row r="32" spans="1:2" ht="25.05" customHeight="1">
-      <c r="A32" s="47" t="s">
+      <c r="A32" s="64" t="s">
         <v>37</v>
       </c>
-      <c r="B32" s="48"/>
+      <c r="B32" s="61"/>
     </row>
     <row r="33" spans="1:3" ht="19.95" customHeight="1">
       <c r="A33" s="27" t="s">
@@ -7457,450 +7470,456 @@
   <dimension ref="A1:C50"/>
   <sheetFormatPr defaultRowHeight="13.8"/>
   <cols>
-    <col min="1" max="1" width="36" style="54" customWidth="1"/>
-    <col min="2" max="2" width="70" style="54" customWidth="1"/>
-    <col min="3" max="3" width="50" style="54" customWidth="1"/>
-    <col min="4" max="16384" width="8.796875" style="54"/>
+    <col min="1" max="1" width="36" style="48" customWidth="1"/>
+    <col min="2" max="2" width="70" style="48" customWidth="1"/>
+    <col min="3" max="3" width="50" style="48" customWidth="1"/>
+    <col min="4" max="16384" width="8.796875" style="48"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="22.35" customHeight="1">
-      <c r="A1" s="52" t="s">
+      <c r="A1" s="59" t="s">
         <v>431</v>
       </c>
-      <c r="B1" s="52"/>
-      <c r="C1" s="53"/>
+      <c r="B1" s="59"/>
+      <c r="C1" s="47"/>
     </row>
     <row r="2" spans="1:3" ht="4.8" customHeight="1">
-      <c r="A2" s="55"/>
-      <c r="B2" s="55"/>
-      <c r="C2" s="53"/>
+      <c r="A2" s="57"/>
+      <c r="B2" s="57"/>
+      <c r="C2" s="47"/>
     </row>
     <row r="3" spans="1:3" ht="16.05" customHeight="1">
       <c r="A3" s="56" t="s">
         <v>1</v>
       </c>
       <c r="B3" s="56"/>
-      <c r="C3" s="53"/>
+      <c r="C3" s="47"/>
     </row>
     <row r="4" spans="1:3" ht="24" customHeight="1">
-      <c r="A4" s="57" t="s">
+      <c r="A4" s="50" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="58" t="s">
+      <c r="B4" s="51" t="s">
         <v>432</v>
       </c>
-      <c r="C4" s="53"/>
+      <c r="C4" s="47"/>
     </row>
     <row r="5" spans="1:3" ht="24" customHeight="1">
-      <c r="A5" s="57" t="s">
+      <c r="A5" s="50" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="58" t="s">
+      <c r="B5" s="51" t="s">
         <v>188</v>
       </c>
-      <c r="C5" s="53"/>
+      <c r="C5" s="47"/>
     </row>
     <row r="6" spans="1:3" ht="24" customHeight="1">
-      <c r="A6" s="57" t="s">
+      <c r="A6" s="50" t="s">
         <v>6</v>
       </c>
       <c r="B6" s="18">
         <v>200</v>
       </c>
-      <c r="C6" s="53"/>
+      <c r="C6" s="47"/>
     </row>
     <row r="7" spans="1:3" ht="24" customHeight="1">
-      <c r="A7" s="57" t="s">
+      <c r="A7" s="50" t="s">
         <v>7</v>
       </c>
       <c r="B7" s="25" t="s">
         <v>120</v>
       </c>
-      <c r="C7" s="53"/>
+      <c r="C7" s="47"/>
     </row>
     <row r="8" spans="1:3" ht="24" customHeight="1">
-      <c r="A8" s="57" t="s">
+      <c r="A8" s="50" t="s">
         <v>9</v>
       </c>
       <c r="B8" s="44" t="s">
         <v>433</v>
       </c>
-      <c r="C8" s="53"/>
+      <c r="C8" s="47"/>
     </row>
     <row r="9" spans="1:3" ht="24" customHeight="1">
-      <c r="A9" s="57" t="s">
+      <c r="A9" s="50" t="s">
         <v>420</v>
       </c>
-      <c r="B9" s="58" t="s">
+      <c r="B9" s="51" t="s">
         <v>443</v>
       </c>
-      <c r="C9" s="53"/>
+      <c r="C9" s="47"/>
     </row>
     <row r="10" spans="1:3" ht="24" customHeight="1">
-      <c r="A10" s="57" t="s">
+      <c r="A10" s="50" t="s">
         <v>11</v>
       </c>
-      <c r="B10" s="58" t="s">
+      <c r="B10" s="51" t="s">
         <v>434</v>
       </c>
-      <c r="C10" s="53"/>
+      <c r="C10" s="47"/>
     </row>
     <row r="11" spans="1:3" ht="4.8" customHeight="1">
-      <c r="A11" s="55"/>
-      <c r="B11" s="55"/>
-      <c r="C11" s="53"/>
+      <c r="A11" s="57"/>
+      <c r="B11" s="57"/>
+      <c r="C11" s="47"/>
     </row>
     <row r="12" spans="1:3" ht="16.05" customHeight="1">
       <c r="A12" s="56" t="s">
         <v>13</v>
       </c>
       <c r="B12" s="56"/>
-      <c r="C12" s="53"/>
+      <c r="C12" s="47"/>
     </row>
     <row r="13" spans="1:3" ht="103.95" customHeight="1">
-      <c r="A13" s="57" t="s">
+      <c r="A13" s="50" t="s">
         <v>14</v>
       </c>
-      <c r="B13" s="58" t="s">
+      <c r="B13" s="51" t="s">
         <v>435</v>
       </c>
-      <c r="C13" s="53"/>
+      <c r="C13" s="47"/>
     </row>
     <row r="14" spans="1:3" ht="4.8" customHeight="1">
-      <c r="A14" s="55"/>
-      <c r="B14" s="55"/>
-      <c r="C14" s="53"/>
+      <c r="A14" s="57"/>
+      <c r="B14" s="57"/>
+      <c r="C14" s="47"/>
     </row>
     <row r="15" spans="1:3" ht="16.05" customHeight="1">
       <c r="A15" s="56" t="s">
         <v>16</v>
       </c>
       <c r="B15" s="56"/>
-      <c r="C15" s="53"/>
+      <c r="C15" s="47"/>
     </row>
     <row r="16" spans="1:3" ht="55.95" customHeight="1">
-      <c r="A16" s="57" t="s">
+      <c r="A16" s="50" t="s">
         <v>17</v>
       </c>
-      <c r="B16" s="58" t="s">
+      <c r="B16" s="51" t="s">
         <v>436</v>
       </c>
-      <c r="C16" s="53"/>
+      <c r="C16" s="47"/>
     </row>
     <row r="17" spans="1:3" ht="79.95" customHeight="1">
-      <c r="A17" s="57" t="s">
+      <c r="A17" s="50" t="s">
         <v>19</v>
       </c>
-      <c r="B17" s="58" t="s">
+      <c r="B17" s="51" t="s">
         <v>437</v>
       </c>
-      <c r="C17" s="53"/>
+      <c r="C17" s="47"/>
     </row>
     <row r="18" spans="1:3" ht="55.95" customHeight="1">
-      <c r="A18" s="57" t="s">
+      <c r="A18" s="50" t="s">
         <v>21</v>
       </c>
-      <c r="B18" s="58" t="s">
+      <c r="B18" s="51" t="s">
         <v>438</v>
       </c>
-      <c r="C18" s="53"/>
+      <c r="C18" s="47"/>
     </row>
     <row r="19" spans="1:3" ht="4.8" customHeight="1">
-      <c r="A19" s="55"/>
-      <c r="B19" s="55"/>
-      <c r="C19" s="53"/>
+      <c r="A19" s="57"/>
+      <c r="B19" s="57"/>
+      <c r="C19" s="47"/>
     </row>
     <row r="20" spans="1:3" ht="16.05" customHeight="1">
       <c r="A20" s="56" t="s">
         <v>23</v>
       </c>
       <c r="B20" s="56"/>
-      <c r="C20" s="53"/>
+      <c r="C20" s="47"/>
     </row>
     <row r="21" spans="1:3" ht="175.95" customHeight="1">
-      <c r="A21" s="57" t="s">
+      <c r="A21" s="50" t="s">
         <v>24</v>
       </c>
-      <c r="B21" s="58" t="s">
+      <c r="B21" s="51" t="s">
         <v>439</v>
       </c>
-      <c r="C21" s="53"/>
+      <c r="C21" s="47"/>
     </row>
     <row r="22" spans="1:3" ht="4.8" customHeight="1">
-      <c r="A22" s="55"/>
-      <c r="B22" s="55"/>
-      <c r="C22" s="53"/>
+      <c r="A22" s="57"/>
+      <c r="B22" s="57"/>
+      <c r="C22" s="47"/>
     </row>
     <row r="23" spans="1:3" ht="16.05" customHeight="1">
       <c r="A23" s="56" t="s">
         <v>26</v>
       </c>
       <c r="B23" s="56"/>
-      <c r="C23" s="53"/>
+      <c r="C23" s="47"/>
     </row>
     <row r="24" spans="1:3" ht="96" customHeight="1">
-      <c r="A24" s="57" t="s">
+      <c r="A24" s="50" t="s">
         <v>27</v>
       </c>
-      <c r="B24" s="58" t="s">
+      <c r="B24" s="51" t="s">
         <v>440</v>
       </c>
-      <c r="C24" s="53"/>
+      <c r="C24" s="47"/>
     </row>
     <row r="25" spans="1:3" ht="103.95" customHeight="1">
-      <c r="A25" s="57" t="s">
+      <c r="A25" s="50" t="s">
         <v>29</v>
       </c>
-      <c r="B25" s="58" t="s">
+      <c r="B25" s="51" t="s">
         <v>441</v>
       </c>
-      <c r="C25" s="53"/>
+      <c r="C25" s="47"/>
     </row>
     <row r="26" spans="1:3" ht="103.95" customHeight="1">
-      <c r="A26" s="57" t="s">
+      <c r="A26" s="50" t="s">
         <v>31</v>
       </c>
-      <c r="B26" s="58" t="s">
+      <c r="B26" s="51" t="s">
         <v>442</v>
       </c>
-      <c r="C26" s="53"/>
+      <c r="C26" s="47"/>
     </row>
     <row r="27" spans="1:3" ht="4.8" customHeight="1">
-      <c r="A27" s="55"/>
-      <c r="B27" s="55"/>
-      <c r="C27" s="53"/>
+      <c r="A27" s="57"/>
+      <c r="B27" s="57"/>
+      <c r="C27" s="47"/>
     </row>
     <row r="28" spans="1:3" ht="16.05" customHeight="1">
       <c r="A28" s="56" t="s">
         <v>33</v>
       </c>
       <c r="B28" s="56"/>
-      <c r="C28" s="53"/>
+      <c r="C28" s="47"/>
     </row>
     <row r="29" spans="1:3" ht="16.05" customHeight="1">
-      <c r="A29" s="57" t="s">
+      <c r="A29" s="50" t="s">
         <v>34</v>
       </c>
       <c r="B29" s="44" t="s">
         <v>445</v>
       </c>
-      <c r="C29" s="53"/>
+      <c r="C29" s="47"/>
     </row>
     <row r="30" spans="1:3" ht="16.05" customHeight="1">
-      <c r="A30" s="57" t="s">
+      <c r="A30" s="50" t="s">
         <v>35</v>
       </c>
       <c r="B30" s="44" t="s">
         <v>444</v>
       </c>
-      <c r="C30" s="53"/>
+      <c r="C30" s="47"/>
     </row>
     <row r="31" spans="1:3" ht="4.8" customHeight="1">
-      <c r="A31" s="55"/>
-      <c r="B31" s="55"/>
-      <c r="C31" s="53"/>
+      <c r="A31" s="57"/>
+      <c r="B31" s="57"/>
+      <c r="C31" s="47"/>
     </row>
     <row r="32" spans="1:3" ht="16.05" customHeight="1">
-      <c r="A32" s="59" t="s">
+      <c r="A32" s="58" t="s">
         <v>37</v>
       </c>
-      <c r="B32" s="59"/>
-      <c r="C32" s="53"/>
+      <c r="B32" s="58"/>
+      <c r="C32" s="47"/>
     </row>
     <row r="33" spans="1:3" ht="16.05" customHeight="1">
-      <c r="A33" s="60" t="s">
+      <c r="A33" s="49" t="s">
         <v>38</v>
       </c>
-      <c r="B33" s="60" t="s">
+      <c r="B33" s="49" t="s">
         <v>39</v>
       </c>
-      <c r="C33" s="60" t="s">
+      <c r="C33" s="49" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="34" spans="1:3" ht="14.4" customHeight="1">
-      <c r="A34" s="61" t="s">
+      <c r="A34" s="52" t="s">
         <v>41</v>
       </c>
-      <c r="B34" s="62" t="s">
+      <c r="B34" s="53" t="s">
         <v>42</v>
       </c>
-      <c r="C34" s="62" t="s">
+      <c r="C34" s="53" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="35" spans="1:3" ht="14.4" customHeight="1">
-      <c r="A35" s="63" t="s">
+      <c r="A35" s="54" t="s">
         <v>44</v>
       </c>
-      <c r="B35" s="64" t="s">
+      <c r="B35" s="55" t="s">
         <v>45</v>
       </c>
-      <c r="C35" s="64" t="s">
+      <c r="C35" s="55" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="36" spans="1:3" ht="14.4" customHeight="1">
-      <c r="A36" s="61" t="s">
+      <c r="A36" s="52" t="s">
         <v>47</v>
       </c>
-      <c r="B36" s="62" t="s">
+      <c r="B36" s="53" t="s">
         <v>48</v>
       </c>
-      <c r="C36" s="62" t="s">
+      <c r="C36" s="53" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="37" spans="1:3" ht="14.4" customHeight="1">
-      <c r="A37" s="63" t="s">
+      <c r="A37" s="54" t="s">
         <v>50</v>
       </c>
-      <c r="B37" s="64" t="s">
+      <c r="B37" s="55" t="s">
         <v>51</v>
       </c>
-      <c r="C37" s="64" t="s">
+      <c r="C37" s="55" t="s">
         <v>52</v>
       </c>
     </row>
     <row r="38" spans="1:3" ht="14.4" customHeight="1">
-      <c r="A38" s="61" t="s">
+      <c r="A38" s="52" t="s">
         <v>53</v>
       </c>
-      <c r="B38" s="62" t="s">
+      <c r="B38" s="53" t="s">
         <v>54</v>
       </c>
-      <c r="C38" s="62" t="s">
+      <c r="C38" s="53" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="39" spans="1:3" ht="14.4" customHeight="1">
-      <c r="A39" s="63" t="s">
+      <c r="A39" s="54" t="s">
         <v>56</v>
       </c>
-      <c r="B39" s="64" t="s">
+      <c r="B39" s="55" t="s">
         <v>57</v>
       </c>
-      <c r="C39" s="64" t="s">
+      <c r="C39" s="55" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="40" spans="1:3" ht="14.4" customHeight="1">
-      <c r="A40" s="61" t="s">
+      <c r="A40" s="52" t="s">
         <v>59</v>
       </c>
-      <c r="B40" s="62" t="s">
+      <c r="B40" s="53" t="s">
         <v>60</v>
       </c>
-      <c r="C40" s="62" t="s">
+      <c r="C40" s="53" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="41" spans="1:3" ht="14.4" customHeight="1">
-      <c r="A41" s="63" t="s">
+      <c r="A41" s="54" t="s">
         <v>62</v>
       </c>
-      <c r="B41" s="64" t="s">
+      <c r="B41" s="55" t="s">
         <v>63</v>
       </c>
-      <c r="C41" s="64" t="s">
+      <c r="C41" s="55" t="s">
         <v>64</v>
       </c>
     </row>
     <row r="42" spans="1:3" ht="14.4" customHeight="1">
-      <c r="A42" s="61" t="s">
+      <c r="A42" s="52" t="s">
         <v>65</v>
       </c>
-      <c r="B42" s="62" t="s">
+      <c r="B42" s="53" t="s">
         <v>66</v>
       </c>
-      <c r="C42" s="62" t="s">
+      <c r="C42" s="53" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="43" spans="1:3" ht="14.4" customHeight="1">
-      <c r="A43" s="63" t="s">
+      <c r="A43" s="54" t="s">
         <v>68</v>
       </c>
-      <c r="B43" s="64" t="s">
+      <c r="B43" s="55" t="s">
         <v>69</v>
       </c>
-      <c r="C43" s="64" t="s">
+      <c r="C43" s="55" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="44" spans="1:3" ht="14.4" customHeight="1">
-      <c r="A44" s="61" t="s">
+      <c r="A44" s="52" t="s">
         <v>71</v>
       </c>
-      <c r="B44" s="62" t="s">
+      <c r="B44" s="53" t="s">
         <v>72</v>
       </c>
-      <c r="C44" s="62" t="s">
+      <c r="C44" s="53" t="s">
         <v>73</v>
       </c>
     </row>
     <row r="45" spans="1:3" ht="14.4" customHeight="1">
-      <c r="A45" s="63" t="s">
+      <c r="A45" s="54" t="s">
         <v>74</v>
       </c>
-      <c r="B45" s="64" t="s">
+      <c r="B45" s="55" t="s">
         <v>75</v>
       </c>
-      <c r="C45" s="64" t="s">
+      <c r="C45" s="55" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="46" spans="1:3" ht="14.4" customHeight="1">
-      <c r="A46" s="61" t="s">
+      <c r="A46" s="52" t="s">
         <v>77</v>
       </c>
-      <c r="B46" s="62" t="s">
+      <c r="B46" s="53" t="s">
         <v>78</v>
       </c>
-      <c r="C46" s="62" t="s">
+      <c r="C46" s="53" t="s">
         <v>79</v>
       </c>
     </row>
     <row r="47" spans="1:3" ht="14.4" customHeight="1">
-      <c r="A47" s="63" t="s">
+      <c r="A47" s="54" t="s">
         <v>80</v>
       </c>
-      <c r="B47" s="64" t="s">
+      <c r="B47" s="55" t="s">
         <v>81</v>
       </c>
-      <c r="C47" s="64" t="s">
+      <c r="C47" s="55" t="s">
         <v>82</v>
       </c>
     </row>
     <row r="48" spans="1:3" ht="14.4" customHeight="1">
-      <c r="A48" s="61" t="s">
+      <c r="A48" s="52" t="s">
         <v>83</v>
       </c>
-      <c r="B48" s="62" t="s">
+      <c r="B48" s="53" t="s">
         <v>84</v>
       </c>
-      <c r="C48" s="62" t="s">
+      <c r="C48" s="53" t="s">
         <v>85</v>
       </c>
     </row>
     <row r="49" spans="1:3" ht="14.4" customHeight="1">
-      <c r="A49" s="63" t="s">
+      <c r="A49" s="54" t="s">
         <v>86</v>
       </c>
-      <c r="B49" s="64" t="s">
+      <c r="B49" s="55" t="s">
         <v>87</v>
       </c>
-      <c r="C49" s="64" t="s">
+      <c r="C49" s="55" t="s">
         <v>88</v>
       </c>
     </row>
     <row r="50" spans="1:3">
-      <c r="A50" s="53"/>
-      <c r="B50" s="53"/>
-      <c r="C50" s="53"/>
+      <c r="A50" s="47"/>
+      <c r="B50" s="47"/>
+      <c r="C50" s="47"/>
     </row>
   </sheetData>
   <mergeCells count="15">
+    <mergeCell ref="A14:B14"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="A3:B3"/>
+    <mergeCell ref="A11:B11"/>
+    <mergeCell ref="A12:B12"/>
     <mergeCell ref="A28:B28"/>
     <mergeCell ref="A31:B31"/>
     <mergeCell ref="A32:B32"/>
@@ -7910,12 +7929,6 @@
     <mergeCell ref="A22:B22"/>
     <mergeCell ref="A23:B23"/>
     <mergeCell ref="A27:B27"/>
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="A3:B3"/>
-    <mergeCell ref="A11:B11"/>
-    <mergeCell ref="A12:B12"/>
-    <mergeCell ref="A14:B14"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="B30" r:id="rId1" xr:uid="{8E46879D-E49B-4394-B81D-ABE38B03AD1F}"/>
@@ -7938,20 +7951,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="30" customHeight="1">
-      <c r="A1" s="49" t="s">
+      <c r="A1" s="62" t="s">
         <v>149</v>
       </c>
-      <c r="B1" s="48"/>
+      <c r="B1" s="61"/>
     </row>
     <row r="2" spans="1:2" ht="6" customHeight="1">
-      <c r="A2" s="48"/>
-      <c r="B2" s="48"/>
+      <c r="A2" s="61"/>
+      <c r="B2" s="61"/>
     </row>
     <row r="3" spans="1:2" ht="30" customHeight="1">
-      <c r="A3" s="50" t="s">
+      <c r="A3" s="63" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="48"/>
+      <c r="B3" s="61"/>
     </row>
     <row r="4" spans="1:2" ht="27.6" customHeight="1">
       <c r="A4" s="17" t="s">
@@ -8010,14 +8023,14 @@
       </c>
     </row>
     <row r="11" spans="1:2">
-      <c r="A11" s="48"/>
-      <c r="B11" s="48"/>
+      <c r="A11" s="61"/>
+      <c r="B11" s="61"/>
     </row>
     <row r="12" spans="1:2" ht="30" customHeight="1">
-      <c r="A12" s="50" t="s">
+      <c r="A12" s="63" t="s">
         <v>13</v>
       </c>
-      <c r="B12" s="48"/>
+      <c r="B12" s="61"/>
     </row>
     <row r="13" spans="1:2" ht="207" customHeight="1">
       <c r="A13" s="17" t="s">
@@ -8028,14 +8041,14 @@
       </c>
     </row>
     <row r="14" spans="1:2">
-      <c r="A14" s="48"/>
-      <c r="B14" s="48"/>
+      <c r="A14" s="61"/>
+      <c r="B14" s="61"/>
     </row>
     <row r="15" spans="1:2" ht="30" customHeight="1">
-      <c r="A15" s="50" t="s">
+      <c r="A15" s="63" t="s">
         <v>16</v>
       </c>
-      <c r="B15" s="48"/>
+      <c r="B15" s="61"/>
     </row>
     <row r="16" spans="1:2" ht="105" customHeight="1">
       <c r="A16" s="17" t="s">
@@ -8062,14 +8075,14 @@
       </c>
     </row>
     <row r="19" spans="1:2">
-      <c r="A19" s="48"/>
-      <c r="B19" s="48"/>
+      <c r="A19" s="61"/>
+      <c r="B19" s="61"/>
     </row>
     <row r="20" spans="1:2" ht="30" customHeight="1">
-      <c r="A20" s="50" t="s">
+      <c r="A20" s="63" t="s">
         <v>23</v>
       </c>
-      <c r="B20" s="48"/>
+      <c r="B20" s="61"/>
     </row>
     <row r="21" spans="1:2" ht="372.6" customHeight="1">
       <c r="A21" s="17" t="s">
@@ -8080,14 +8093,14 @@
       </c>
     </row>
     <row r="22" spans="1:2">
-      <c r="A22" s="48"/>
-      <c r="B22" s="48"/>
+      <c r="A22" s="61"/>
+      <c r="B22" s="61"/>
     </row>
     <row r="23" spans="1:2" ht="30" customHeight="1">
-      <c r="A23" s="50" t="s">
+      <c r="A23" s="63" t="s">
         <v>26</v>
       </c>
-      <c r="B23" s="48"/>
+      <c r="B23" s="61"/>
     </row>
     <row r="24" spans="1:2" ht="151.80000000000001" customHeight="1">
       <c r="A24" s="17" t="s">
@@ -8114,14 +8127,14 @@
       </c>
     </row>
     <row r="27" spans="1:2">
-      <c r="A27" s="48"/>
-      <c r="B27" s="48"/>
+      <c r="A27" s="61"/>
+      <c r="B27" s="61"/>
     </row>
     <row r="28" spans="1:2" ht="30" customHeight="1">
-      <c r="A28" s="50" t="s">
+      <c r="A28" s="63" t="s">
         <v>33</v>
       </c>
-      <c r="B28" s="48"/>
+      <c r="B28" s="61"/>
     </row>
     <row r="29" spans="1:2" ht="18" customHeight="1">
       <c r="A29" s="17" t="s">
@@ -8140,14 +8153,14 @@
       </c>
     </row>
     <row r="31" spans="1:2">
-      <c r="A31" s="48"/>
-      <c r="B31" s="48"/>
+      <c r="A31" s="61"/>
+      <c r="B31" s="61"/>
     </row>
     <row r="32" spans="1:2" ht="25.05" customHeight="1">
-      <c r="A32" s="47" t="s">
+      <c r="A32" s="64" t="s">
         <v>37</v>
       </c>
-      <c r="B32" s="48"/>
+      <c r="B32" s="61"/>
     </row>
     <row r="33" spans="1:3" ht="19.95" customHeight="1">
       <c r="A33" s="20" t="s">
@@ -36644,20 +36657,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="30" customHeight="1">
-      <c r="A1" s="49" t="s">
+      <c r="A1" s="62" t="s">
         <v>163</v>
       </c>
-      <c r="B1" s="48"/>
+      <c r="B1" s="61"/>
     </row>
     <row r="2" spans="1:2" ht="6" customHeight="1">
-      <c r="A2" s="48"/>
-      <c r="B2" s="48"/>
+      <c r="A2" s="61"/>
+      <c r="B2" s="61"/>
     </row>
     <row r="3" spans="1:2" ht="30" customHeight="1">
-      <c r="A3" s="50" t="s">
+      <c r="A3" s="63" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="48"/>
+      <c r="B3" s="61"/>
     </row>
     <row r="4" spans="1:2" ht="18" customHeight="1">
       <c r="A4" s="17" t="s">
@@ -36716,14 +36729,14 @@
       </c>
     </row>
     <row r="11" spans="1:2">
-      <c r="A11" s="48"/>
-      <c r="B11" s="48"/>
+      <c r="A11" s="61"/>
+      <c r="B11" s="61"/>
     </row>
     <row r="12" spans="1:2" ht="30" customHeight="1">
-      <c r="A12" s="50" t="s">
+      <c r="A12" s="63" t="s">
         <v>13</v>
       </c>
-      <c r="B12" s="48"/>
+      <c r="B12" s="61"/>
     </row>
     <row r="13" spans="1:2" ht="248.4" customHeight="1">
       <c r="A13" s="17" t="s">
@@ -36734,14 +36747,14 @@
       </c>
     </row>
     <row r="14" spans="1:2">
-      <c r="A14" s="48"/>
-      <c r="B14" s="48"/>
+      <c r="A14" s="61"/>
+      <c r="B14" s="61"/>
     </row>
     <row r="15" spans="1:2" ht="30" customHeight="1">
-      <c r="A15" s="50" t="s">
+      <c r="A15" s="63" t="s">
         <v>16</v>
       </c>
-      <c r="B15" s="48"/>
+      <c r="B15" s="61"/>
     </row>
     <row r="16" spans="1:2" ht="96.6" customHeight="1">
       <c r="A16" s="17" t="s">
@@ -36768,14 +36781,14 @@
       </c>
     </row>
     <row r="19" spans="1:2">
-      <c r="A19" s="48"/>
-      <c r="B19" s="48"/>
+      <c r="A19" s="61"/>
+      <c r="B19" s="61"/>
     </row>
     <row r="20" spans="1:2">
-      <c r="A20" s="50" t="s">
+      <c r="A20" s="63" t="s">
         <v>23</v>
       </c>
-      <c r="B20" s="48"/>
+      <c r="B20" s="61"/>
     </row>
     <row r="21" spans="1:2" ht="400.2" customHeight="1">
       <c r="A21" s="17" t="s">
@@ -36786,14 +36799,14 @@
       </c>
     </row>
     <row r="22" spans="1:2" ht="6" customHeight="1">
-      <c r="A22" s="48"/>
-      <c r="B22" s="48"/>
+      <c r="A22" s="61"/>
+      <c r="B22" s="61"/>
     </row>
     <row r="23" spans="1:2" ht="30" customHeight="1">
-      <c r="A23" s="50" t="s">
+      <c r="A23" s="63" t="s">
         <v>26</v>
       </c>
-      <c r="B23" s="48"/>
+      <c r="B23" s="61"/>
     </row>
     <row r="24" spans="1:2" ht="138" customHeight="1">
       <c r="A24" s="17" t="s">
@@ -36820,14 +36833,14 @@
       </c>
     </row>
     <row r="27" spans="1:2">
-      <c r="A27" s="48"/>
-      <c r="B27" s="48"/>
+      <c r="A27" s="61"/>
+      <c r="B27" s="61"/>
     </row>
     <row r="28" spans="1:2" ht="30" customHeight="1">
-      <c r="A28" s="50" t="s">
+      <c r="A28" s="63" t="s">
         <v>33</v>
       </c>
-      <c r="B28" s="48"/>
+      <c r="B28" s="61"/>
     </row>
     <row r="29" spans="1:2" ht="18" customHeight="1">
       <c r="A29" s="17" t="s">
@@ -36846,14 +36859,14 @@
       </c>
     </row>
     <row r="31" spans="1:2" ht="6" customHeight="1">
-      <c r="A31" s="48"/>
-      <c r="B31" s="48"/>
+      <c r="A31" s="61"/>
+      <c r="B31" s="61"/>
     </row>
     <row r="32" spans="1:2" ht="25.05" customHeight="1">
-      <c r="A32" s="47" t="s">
+      <c r="A32" s="64" t="s">
         <v>37</v>
       </c>
-      <c r="B32" s="48"/>
+      <c r="B32" s="61"/>
     </row>
     <row r="33" spans="1:3" ht="19.95" customHeight="1">
       <c r="A33" s="20" t="s">
@@ -37080,20 +37093,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="30" customHeight="1">
-      <c r="A1" s="49" t="s">
+      <c r="A1" s="62" t="s">
         <v>176</v>
       </c>
-      <c r="B1" s="48"/>
+      <c r="B1" s="61"/>
     </row>
     <row r="2" spans="1:2" ht="6" customHeight="1">
-      <c r="A2" s="48"/>
-      <c r="B2" s="48"/>
+      <c r="A2" s="61"/>
+      <c r="B2" s="61"/>
     </row>
     <row r="3" spans="1:2" ht="30" customHeight="1">
-      <c r="A3" s="50" t="s">
+      <c r="A3" s="63" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="48"/>
+      <c r="B3" s="61"/>
     </row>
     <row r="4" spans="1:2" ht="18" customHeight="1">
       <c r="A4" s="17" t="s">
@@ -37152,14 +37165,14 @@
       </c>
     </row>
     <row r="11" spans="1:2">
-      <c r="A11" s="48"/>
-      <c r="B11" s="48"/>
+      <c r="A11" s="61"/>
+      <c r="B11" s="61"/>
     </row>
     <row r="12" spans="1:2" ht="30" customHeight="1">
-      <c r="A12" s="50" t="s">
+      <c r="A12" s="63" t="s">
         <v>13</v>
       </c>
-      <c r="B12" s="48"/>
+      <c r="B12" s="61"/>
     </row>
     <row r="13" spans="1:2" ht="345" customHeight="1">
       <c r="A13" s="17" t="s">
@@ -37170,14 +37183,14 @@
       </c>
     </row>
     <row r="14" spans="1:2">
-      <c r="A14" s="48"/>
-      <c r="B14" s="48"/>
+      <c r="A14" s="61"/>
+      <c r="B14" s="61"/>
     </row>
     <row r="15" spans="1:2" ht="30" customHeight="1">
-      <c r="A15" s="50" t="s">
+      <c r="A15" s="63" t="s">
         <v>16</v>
       </c>
-      <c r="B15" s="48"/>
+      <c r="B15" s="61"/>
     </row>
     <row r="16" spans="1:2" ht="105" customHeight="1">
       <c r="A16" s="17" t="s">
@@ -37204,14 +37217,14 @@
       </c>
     </row>
     <row r="19" spans="1:2">
-      <c r="A19" s="48"/>
-      <c r="B19" s="48"/>
+      <c r="A19" s="61"/>
+      <c r="B19" s="61"/>
     </row>
     <row r="20" spans="1:2" ht="30" customHeight="1">
-      <c r="A20" s="50" t="s">
+      <c r="A20" s="63" t="s">
         <v>23</v>
       </c>
-      <c r="B20" s="48"/>
+      <c r="B20" s="61"/>
     </row>
     <row r="21" spans="1:2" ht="409.6" customHeight="1">
       <c r="A21" s="17" t="s">
@@ -37222,14 +37235,14 @@
       </c>
     </row>
     <row r="22" spans="1:2">
-      <c r="A22" s="48"/>
-      <c r="B22" s="48"/>
+      <c r="A22" s="61"/>
+      <c r="B22" s="61"/>
     </row>
     <row r="23" spans="1:2" ht="30" customHeight="1">
-      <c r="A23" s="50" t="s">
+      <c r="A23" s="63" t="s">
         <v>26</v>
       </c>
-      <c r="B23" s="48"/>
+      <c r="B23" s="61"/>
     </row>
     <row r="24" spans="1:2" ht="135" customHeight="1">
       <c r="A24" s="17" t="s">
@@ -37256,14 +37269,14 @@
       </c>
     </row>
     <row r="27" spans="1:2">
-      <c r="A27" s="48"/>
-      <c r="B27" s="48"/>
+      <c r="A27" s="61"/>
+      <c r="B27" s="61"/>
     </row>
     <row r="28" spans="1:2" ht="30" customHeight="1">
-      <c r="A28" s="50" t="s">
+      <c r="A28" s="63" t="s">
         <v>33</v>
       </c>
-      <c r="B28" s="48"/>
+      <c r="B28" s="61"/>
     </row>
     <row r="29" spans="1:2" ht="18" customHeight="1">
       <c r="A29" s="17" t="s">
@@ -37282,14 +37295,14 @@
       </c>
     </row>
     <row r="31" spans="1:2" ht="6" customHeight="1">
-      <c r="A31" s="48"/>
-      <c r="B31" s="48"/>
+      <c r="A31" s="61"/>
+      <c r="B31" s="61"/>
     </row>
     <row r="32" spans="1:2" ht="25.05" customHeight="1">
-      <c r="A32" s="47" t="s">
+      <c r="A32" s="64" t="s">
         <v>37</v>
       </c>
-      <c r="B32" s="48"/>
+      <c r="B32" s="61"/>
     </row>
     <row r="33" spans="1:3" ht="19.95" customHeight="1">
       <c r="A33" s="20" t="s">
@@ -37516,20 +37529,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="30" customHeight="1">
-      <c r="A1" s="49" t="s">
+      <c r="A1" s="62" t="s">
         <v>186</v>
       </c>
-      <c r="B1" s="48"/>
+      <c r="B1" s="61"/>
     </row>
     <row r="2" spans="1:2">
-      <c r="A2" s="48"/>
-      <c r="B2" s="48"/>
+      <c r="A2" s="61"/>
+      <c r="B2" s="61"/>
     </row>
     <row r="3" spans="1:2" ht="30" customHeight="1">
-      <c r="A3" s="50" t="s">
+      <c r="A3" s="63" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="48"/>
+      <c r="B3" s="61"/>
     </row>
     <row r="4" spans="1:2" ht="15" customHeight="1">
       <c r="A4" s="17" t="s">
@@ -37588,14 +37601,14 @@
       </c>
     </row>
     <row r="11" spans="1:2">
-      <c r="A11" s="48"/>
-      <c r="B11" s="48"/>
+      <c r="A11" s="61"/>
+      <c r="B11" s="61"/>
     </row>
     <row r="12" spans="1:2" ht="30" customHeight="1">
-      <c r="A12" s="50" t="s">
+      <c r="A12" s="63" t="s">
         <v>13</v>
       </c>
-      <c r="B12" s="48"/>
+      <c r="B12" s="61"/>
     </row>
     <row r="13" spans="1:2" ht="207" customHeight="1">
       <c r="A13" s="17" t="s">
@@ -37606,14 +37619,14 @@
       </c>
     </row>
     <row r="14" spans="1:2">
-      <c r="A14" s="48"/>
-      <c r="B14" s="48"/>
+      <c r="A14" s="61"/>
+      <c r="B14" s="61"/>
     </row>
     <row r="15" spans="1:2" ht="30" customHeight="1">
-      <c r="A15" s="50" t="s">
+      <c r="A15" s="63" t="s">
         <v>16</v>
       </c>
-      <c r="B15" s="48"/>
+      <c r="B15" s="61"/>
     </row>
     <row r="16" spans="1:2" ht="110.4" customHeight="1">
       <c r="A16" s="17" t="s">
@@ -37640,14 +37653,14 @@
       </c>
     </row>
     <row r="19" spans="1:2">
-      <c r="A19" s="48"/>
-      <c r="B19" s="48"/>
+      <c r="A19" s="61"/>
+      <c r="B19" s="61"/>
     </row>
     <row r="20" spans="1:2" ht="30" customHeight="1">
-      <c r="A20" s="50" t="s">
+      <c r="A20" s="63" t="s">
         <v>23</v>
       </c>
-      <c r="B20" s="48"/>
+      <c r="B20" s="61"/>
     </row>
     <row r="21" spans="1:2" ht="303.60000000000002" customHeight="1">
       <c r="A21" s="17" t="s">
@@ -37658,14 +37671,14 @@
       </c>
     </row>
     <row r="22" spans="1:2">
-      <c r="A22" s="48"/>
-      <c r="B22" s="48"/>
+      <c r="A22" s="61"/>
+      <c r="B22" s="61"/>
     </row>
     <row r="23" spans="1:2" ht="30" customHeight="1">
-      <c r="A23" s="50" t="s">
+      <c r="A23" s="63" t="s">
         <v>26</v>
       </c>
-      <c r="B23" s="48"/>
+      <c r="B23" s="61"/>
     </row>
     <row r="24" spans="1:2" ht="82.8" customHeight="1">
       <c r="A24" s="17" t="s">
@@ -37692,14 +37705,14 @@
       </c>
     </row>
     <row r="27" spans="1:2">
-      <c r="A27" s="48"/>
-      <c r="B27" s="48"/>
+      <c r="A27" s="61"/>
+      <c r="B27" s="61"/>
     </row>
     <row r="28" spans="1:2" ht="30" customHeight="1">
-      <c r="A28" s="50" t="s">
+      <c r="A28" s="63" t="s">
         <v>33</v>
       </c>
-      <c r="B28" s="48"/>
+      <c r="B28" s="61"/>
     </row>
     <row r="29" spans="1:2" ht="15" customHeight="1">
       <c r="A29" s="17" t="s">
@@ -37718,14 +37731,14 @@
       </c>
     </row>
     <row r="31" spans="1:2">
-      <c r="A31" s="48"/>
-      <c r="B31" s="48"/>
+      <c r="A31" s="61"/>
+      <c r="B31" s="61"/>
     </row>
     <row r="32" spans="1:2" ht="25.05" customHeight="1">
-      <c r="A32" s="47" t="s">
+      <c r="A32" s="64" t="s">
         <v>37</v>
       </c>
-      <c r="B32" s="48"/>
+      <c r="B32" s="61"/>
     </row>
     <row r="33" spans="1:3" ht="19.95" customHeight="1">
       <c r="A33" s="20" t="s">
@@ -37952,20 +37965,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="30" customHeight="1">
-      <c r="A1" s="49" t="s">
+      <c r="A1" s="62" t="s">
         <v>201</v>
       </c>
-      <c r="B1" s="48"/>
+      <c r="B1" s="61"/>
     </row>
     <row r="2" spans="1:2" ht="6" customHeight="1">
-      <c r="A2" s="48"/>
-      <c r="B2" s="48"/>
+      <c r="A2" s="61"/>
+      <c r="B2" s="61"/>
     </row>
     <row r="3" spans="1:2" ht="30" customHeight="1">
-      <c r="A3" s="50" t="s">
+      <c r="A3" s="63" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="48"/>
+      <c r="B3" s="61"/>
     </row>
     <row r="4" spans="1:2" ht="18" customHeight="1">
       <c r="A4" s="17" t="s">
@@ -38024,14 +38037,14 @@
       </c>
     </row>
     <row r="11" spans="1:2" ht="6" customHeight="1">
-      <c r="A11" s="48"/>
-      <c r="B11" s="48"/>
+      <c r="A11" s="61"/>
+      <c r="B11" s="61"/>
     </row>
     <row r="12" spans="1:2" ht="30" customHeight="1">
-      <c r="A12" s="50" t="s">
+      <c r="A12" s="63" t="s">
         <v>13</v>
       </c>
-      <c r="B12" s="48"/>
+      <c r="B12" s="61"/>
     </row>
     <row r="13" spans="1:2" ht="358.8" customHeight="1">
       <c r="A13" s="17" t="s">
@@ -38042,14 +38055,14 @@
       </c>
     </row>
     <row r="14" spans="1:2">
-      <c r="A14" s="48"/>
-      <c r="B14" s="48"/>
+      <c r="A14" s="61"/>
+      <c r="B14" s="61"/>
     </row>
     <row r="15" spans="1:2" ht="30" customHeight="1">
-      <c r="A15" s="50" t="s">
+      <c r="A15" s="63" t="s">
         <v>16</v>
       </c>
-      <c r="B15" s="48"/>
+      <c r="B15" s="61"/>
     </row>
     <row r="16" spans="1:2" ht="138" customHeight="1">
       <c r="A16" s="17" t="s">
@@ -38076,14 +38089,14 @@
       </c>
     </row>
     <row r="19" spans="1:2" ht="6" customHeight="1">
-      <c r="A19" s="48"/>
-      <c r="B19" s="48"/>
+      <c r="A19" s="61"/>
+      <c r="B19" s="61"/>
     </row>
     <row r="20" spans="1:2" ht="30" customHeight="1">
-      <c r="A20" s="50" t="s">
+      <c r="A20" s="63" t="s">
         <v>23</v>
       </c>
-      <c r="B20" s="48"/>
+      <c r="B20" s="61"/>
     </row>
     <row r="21" spans="1:2" ht="358.8" customHeight="1">
       <c r="A21" s="17" t="s">
@@ -38094,14 +38107,14 @@
       </c>
     </row>
     <row r="22" spans="1:2" ht="6" customHeight="1">
-      <c r="A22" s="48"/>
-      <c r="B22" s="48"/>
+      <c r="A22" s="61"/>
+      <c r="B22" s="61"/>
     </row>
     <row r="23" spans="1:2" ht="30" customHeight="1">
-      <c r="A23" s="50" t="s">
+      <c r="A23" s="63" t="s">
         <v>26</v>
       </c>
-      <c r="B23" s="48"/>
+      <c r="B23" s="61"/>
     </row>
     <row r="24" spans="1:2" ht="90" customHeight="1">
       <c r="A24" s="17" t="s">
@@ -38128,14 +38141,14 @@
       </c>
     </row>
     <row r="27" spans="1:2" ht="6" customHeight="1">
-      <c r="A27" s="48"/>
-      <c r="B27" s="48"/>
+      <c r="A27" s="61"/>
+      <c r="B27" s="61"/>
     </row>
     <row r="28" spans="1:2" ht="30" customHeight="1">
-      <c r="A28" s="50" t="s">
+      <c r="A28" s="63" t="s">
         <v>33</v>
       </c>
-      <c r="B28" s="48"/>
+      <c r="B28" s="61"/>
     </row>
     <row r="29" spans="1:2" ht="18" customHeight="1">
       <c r="A29" s="17" t="s">
@@ -38154,14 +38167,14 @@
       </c>
     </row>
     <row r="31" spans="1:2" ht="6" customHeight="1">
-      <c r="A31" s="48"/>
-      <c r="B31" s="48"/>
+      <c r="A31" s="61"/>
+      <c r="B31" s="61"/>
     </row>
     <row r="32" spans="1:2" ht="25.05" customHeight="1">
-      <c r="A32" s="47" t="s">
+      <c r="A32" s="64" t="s">
         <v>37</v>
       </c>
-      <c r="B32" s="48"/>
+      <c r="B32" s="61"/>
     </row>
     <row r="33" spans="1:3" ht="19.95" customHeight="1">
       <c r="A33" s="20" t="s">
@@ -38389,20 +38402,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="30" customHeight="1">
-      <c r="A1" s="49" t="s">
+      <c r="A1" s="62" t="s">
         <v>216</v>
       </c>
-      <c r="B1" s="48"/>
+      <c r="B1" s="61"/>
     </row>
     <row r="2" spans="1:2" ht="6" customHeight="1">
-      <c r="A2" s="48"/>
-      <c r="B2" s="48"/>
+      <c r="A2" s="61"/>
+      <c r="B2" s="61"/>
     </row>
     <row r="3" spans="1:2" ht="30" customHeight="1">
-      <c r="A3" s="50" t="s">
+      <c r="A3" s="63" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="48"/>
+      <c r="B3" s="61"/>
     </row>
     <row r="4" spans="1:2" ht="18" customHeight="1">
       <c r="A4" s="17" t="s">
@@ -38461,14 +38474,14 @@
       </c>
     </row>
     <row r="11" spans="1:2" ht="6" customHeight="1">
-      <c r="A11" s="48"/>
-      <c r="B11" s="48"/>
+      <c r="A11" s="61"/>
+      <c r="B11" s="61"/>
     </row>
     <row r="12" spans="1:2" ht="30" customHeight="1">
-      <c r="A12" s="50" t="s">
+      <c r="A12" s="63" t="s">
         <v>13</v>
       </c>
-      <c r="B12" s="48"/>
+      <c r="B12" s="61"/>
     </row>
     <row r="13" spans="1:2" ht="317.39999999999998" customHeight="1">
       <c r="A13" s="17" t="s">
@@ -38479,14 +38492,14 @@
       </c>
     </row>
     <row r="14" spans="1:2" ht="6" customHeight="1">
-      <c r="A14" s="48"/>
-      <c r="B14" s="48"/>
+      <c r="A14" s="61"/>
+      <c r="B14" s="61"/>
     </row>
     <row r="15" spans="1:2" ht="30" customHeight="1">
-      <c r="A15" s="50" t="s">
+      <c r="A15" s="63" t="s">
         <v>16</v>
       </c>
-      <c r="B15" s="48"/>
+      <c r="B15" s="61"/>
     </row>
     <row r="16" spans="1:2" ht="105" customHeight="1">
       <c r="A16" s="17" t="s">
@@ -38513,14 +38526,14 @@
       </c>
     </row>
     <row r="19" spans="1:2" ht="6" customHeight="1">
-      <c r="A19" s="48"/>
-      <c r="B19" s="48"/>
+      <c r="A19" s="61"/>
+      <c r="B19" s="61"/>
     </row>
     <row r="20" spans="1:2" ht="30" customHeight="1">
-      <c r="A20" s="50" t="s">
+      <c r="A20" s="63" t="s">
         <v>23</v>
       </c>
-      <c r="B20" s="48"/>
+      <c r="B20" s="61"/>
     </row>
     <row r="21" spans="1:2" ht="372.6" customHeight="1">
       <c r="A21" s="17" t="s">
@@ -38531,14 +38544,14 @@
       </c>
     </row>
     <row r="22" spans="1:2" ht="6" customHeight="1">
-      <c r="A22" s="48"/>
-      <c r="B22" s="48"/>
+      <c r="A22" s="61"/>
+      <c r="B22" s="61"/>
     </row>
     <row r="23" spans="1:2" ht="30" customHeight="1">
-      <c r="A23" s="50" t="s">
+      <c r="A23" s="63" t="s">
         <v>26</v>
       </c>
-      <c r="B23" s="48"/>
+      <c r="B23" s="61"/>
     </row>
     <row r="24" spans="1:2" ht="151.80000000000001" customHeight="1">
       <c r="A24" s="17" t="s">
@@ -38563,14 +38576,14 @@
       <c r="B26" s="18"/>
     </row>
     <row r="27" spans="1:2">
-      <c r="A27" s="48"/>
-      <c r="B27" s="48"/>
+      <c r="A27" s="61"/>
+      <c r="B27" s="61"/>
     </row>
     <row r="28" spans="1:2" ht="30" customHeight="1">
-      <c r="A28" s="50" t="s">
+      <c r="A28" s="63" t="s">
         <v>33</v>
       </c>
-      <c r="B28" s="48"/>
+      <c r="B28" s="61"/>
     </row>
     <row r="29" spans="1:2" ht="18" customHeight="1">
       <c r="A29" s="17" t="s">
@@ -38589,14 +38602,14 @@
       </c>
     </row>
     <row r="31" spans="1:2" ht="6" customHeight="1">
-      <c r="A31" s="48"/>
-      <c r="B31" s="48"/>
+      <c r="A31" s="61"/>
+      <c r="B31" s="61"/>
     </row>
     <row r="32" spans="1:2" ht="25.05" customHeight="1">
-      <c r="A32" s="47" t="s">
+      <c r="A32" s="64" t="s">
         <v>37</v>
       </c>
-      <c r="B32" s="48"/>
+      <c r="B32" s="61"/>
     </row>
     <row r="33" spans="1:3" ht="19.95" customHeight="1">
       <c r="A33" s="20" t="s">
@@ -38823,20 +38836,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="30" customHeight="1">
-      <c r="A1" s="49" t="s">
+      <c r="A1" s="62" t="s">
         <v>228</v>
       </c>
-      <c r="B1" s="48"/>
+      <c r="B1" s="61"/>
     </row>
     <row r="2" spans="1:2" ht="6" customHeight="1">
-      <c r="A2" s="48"/>
-      <c r="B2" s="48"/>
+      <c r="A2" s="61"/>
+      <c r="B2" s="61"/>
     </row>
     <row r="3" spans="1:2" ht="30" customHeight="1">
-      <c r="A3" s="50" t="s">
+      <c r="A3" s="63" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="48"/>
+      <c r="B3" s="61"/>
     </row>
     <row r="4" spans="1:2" ht="18" customHeight="1">
       <c r="A4" s="17" t="s">
@@ -38895,14 +38908,14 @@
       </c>
     </row>
     <row r="11" spans="1:2" ht="6" customHeight="1">
-      <c r="A11" s="48"/>
-      <c r="B11" s="48"/>
+      <c r="A11" s="61"/>
+      <c r="B11" s="61"/>
     </row>
     <row r="12" spans="1:2" ht="30" customHeight="1">
-      <c r="A12" s="50" t="s">
+      <c r="A12" s="63" t="s">
         <v>13</v>
       </c>
-      <c r="B12" s="48"/>
+      <c r="B12" s="61"/>
     </row>
     <row r="13" spans="1:2" ht="207" customHeight="1">
       <c r="A13" s="17" t="s">
@@ -38913,14 +38926,14 @@
       </c>
     </row>
     <row r="14" spans="1:2" ht="6" customHeight="1">
-      <c r="A14" s="48"/>
-      <c r="B14" s="48"/>
+      <c r="A14" s="61"/>
+      <c r="B14" s="61"/>
     </row>
     <row r="15" spans="1:2" ht="30" customHeight="1">
-      <c r="A15" s="50" t="s">
+      <c r="A15" s="63" t="s">
         <v>16</v>
       </c>
-      <c r="B15" s="48"/>
+      <c r="B15" s="61"/>
     </row>
     <row r="16" spans="1:2" ht="110.4" customHeight="1">
       <c r="A16" s="17" t="s">
@@ -38947,14 +38960,14 @@
       </c>
     </row>
     <row r="19" spans="1:2" ht="6" customHeight="1">
-      <c r="A19" s="48"/>
-      <c r="B19" s="48"/>
+      <c r="A19" s="61"/>
+      <c r="B19" s="61"/>
     </row>
     <row r="20" spans="1:2" ht="30" customHeight="1">
-      <c r="A20" s="50" t="s">
+      <c r="A20" s="63" t="s">
         <v>23</v>
       </c>
-      <c r="B20" s="48"/>
+      <c r="B20" s="61"/>
     </row>
     <row r="21" spans="1:2" ht="409.6" customHeight="1">
       <c r="A21" s="17" t="s">
@@ -38965,14 +38978,14 @@
       </c>
     </row>
     <row r="22" spans="1:2" ht="6" customHeight="1">
-      <c r="A22" s="48"/>
-      <c r="B22" s="48"/>
+      <c r="A22" s="61"/>
+      <c r="B22" s="61"/>
     </row>
     <row r="23" spans="1:2" ht="30" customHeight="1">
-      <c r="A23" s="50" t="s">
+      <c r="A23" s="63" t="s">
         <v>26</v>
       </c>
-      <c r="B23" s="48"/>
+      <c r="B23" s="61"/>
     </row>
     <row r="24" spans="1:2" ht="110.4" customHeight="1">
       <c r="A24" s="17" t="s">
@@ -38999,14 +39012,14 @@
       </c>
     </row>
     <row r="27" spans="1:2" ht="6" customHeight="1">
-      <c r="A27" s="48"/>
-      <c r="B27" s="48"/>
+      <c r="A27" s="61"/>
+      <c r="B27" s="61"/>
     </row>
     <row r="28" spans="1:2" ht="30" customHeight="1">
-      <c r="A28" s="50" t="s">
+      <c r="A28" s="63" t="s">
         <v>33</v>
       </c>
-      <c r="B28" s="48"/>
+      <c r="B28" s="61"/>
     </row>
     <row r="29" spans="1:2" ht="18" customHeight="1">
       <c r="A29" s="17" t="s">
@@ -39025,14 +39038,14 @@
       </c>
     </row>
     <row r="31" spans="1:2" ht="6" customHeight="1">
-      <c r="A31" s="48"/>
-      <c r="B31" s="48"/>
+      <c r="A31" s="61"/>
+      <c r="B31" s="61"/>
     </row>
     <row r="32" spans="1:2" ht="25.05" customHeight="1">
-      <c r="A32" s="47" t="s">
+      <c r="A32" s="64" t="s">
         <v>37</v>
       </c>
-      <c r="B32" s="48"/>
+      <c r="B32" s="61"/>
     </row>
     <row r="33" spans="1:3" ht="19.95" customHeight="1">
       <c r="A33" s="20" t="s">
@@ -39260,20 +39273,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="30" customHeight="1">
-      <c r="A1" s="49" t="s">
+      <c r="A1" s="62" t="s">
         <v>243</v>
       </c>
-      <c r="B1" s="48"/>
+      <c r="B1" s="61"/>
     </row>
     <row r="2" spans="1:2" ht="6" customHeight="1">
-      <c r="A2" s="48"/>
-      <c r="B2" s="48"/>
+      <c r="A2" s="61"/>
+      <c r="B2" s="61"/>
     </row>
     <row r="3" spans="1:2" ht="30" customHeight="1">
-      <c r="A3" s="50" t="s">
+      <c r="A3" s="63" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="48"/>
+      <c r="B3" s="61"/>
     </row>
     <row r="4" spans="1:2" ht="18" customHeight="1">
       <c r="A4" s="17" t="s">
@@ -39340,14 +39353,14 @@
       </c>
     </row>
     <row r="12" spans="1:2" ht="6" customHeight="1">
-      <c r="A12" s="48"/>
-      <c r="B12" s="48"/>
+      <c r="A12" s="61"/>
+      <c r="B12" s="61"/>
     </row>
     <row r="13" spans="1:2" ht="30" customHeight="1">
-      <c r="A13" s="50" t="s">
+      <c r="A13" s="63" t="s">
         <v>13</v>
       </c>
-      <c r="B13" s="48"/>
+      <c r="B13" s="61"/>
     </row>
     <row r="14" spans="1:2" ht="193.2" customHeight="1">
       <c r="A14" s="17" t="s">
@@ -39358,14 +39371,14 @@
       </c>
     </row>
     <row r="15" spans="1:2" ht="6" customHeight="1">
-      <c r="A15" s="48"/>
-      <c r="B15" s="48"/>
+      <c r="A15" s="61"/>
+      <c r="B15" s="61"/>
     </row>
     <row r="16" spans="1:2" ht="30" customHeight="1">
-      <c r="A16" s="50" t="s">
+      <c r="A16" s="63" t="s">
         <v>16</v>
       </c>
-      <c r="B16" s="48"/>
+      <c r="B16" s="61"/>
     </row>
     <row r="17" spans="1:2" ht="96.6" customHeight="1">
       <c r="A17" s="17" t="s">
@@ -39392,14 +39405,14 @@
       </c>
     </row>
     <row r="20" spans="1:2" ht="6" customHeight="1">
-      <c r="A20" s="48"/>
-      <c r="B20" s="48"/>
+      <c r="A20" s="61"/>
+      <c r="B20" s="61"/>
     </row>
     <row r="21" spans="1:2" ht="30" customHeight="1">
-      <c r="A21" s="50" t="s">
+      <c r="A21" s="63" t="s">
         <v>23</v>
       </c>
-      <c r="B21" s="48"/>
+      <c r="B21" s="61"/>
     </row>
     <row r="22" spans="1:2" ht="409.6" customHeight="1">
       <c r="A22" s="17" t="s">
@@ -39410,14 +39423,14 @@
       </c>
     </row>
     <row r="23" spans="1:2" ht="6" customHeight="1">
-      <c r="A23" s="48"/>
-      <c r="B23" s="48"/>
+      <c r="A23" s="61"/>
+      <c r="B23" s="61"/>
     </row>
     <row r="24" spans="1:2" ht="30" customHeight="1">
-      <c r="A24" s="50" t="s">
+      <c r="A24" s="63" t="s">
         <v>26</v>
       </c>
-      <c r="B24" s="48"/>
+      <c r="B24" s="61"/>
     </row>
     <row r="25" spans="1:2" ht="151.80000000000001" customHeight="1">
       <c r="A25" s="17" t="s">
@@ -39444,14 +39457,14 @@
       </c>
     </row>
     <row r="28" spans="1:2" ht="6" customHeight="1">
-      <c r="A28" s="48"/>
-      <c r="B28" s="48"/>
+      <c r="A28" s="61"/>
+      <c r="B28" s="61"/>
     </row>
     <row r="29" spans="1:2" ht="30" customHeight="1">
-      <c r="A29" s="50" t="s">
+      <c r="A29" s="63" t="s">
         <v>33</v>
       </c>
-      <c r="B29" s="48"/>
+      <c r="B29" s="61"/>
     </row>
     <row r="30" spans="1:2" ht="18" customHeight="1">
       <c r="A30" s="17" t="s">
@@ -39470,14 +39483,14 @@
       </c>
     </row>
     <row r="32" spans="1:2" ht="6" customHeight="1">
-      <c r="A32" s="48"/>
-      <c r="B32" s="48"/>
+      <c r="A32" s="61"/>
+      <c r="B32" s="61"/>
     </row>
     <row r="33" spans="1:3" ht="25.05" customHeight="1">
-      <c r="A33" s="47" t="s">
+      <c r="A33" s="64" t="s">
         <v>37</v>
       </c>
-      <c r="B33" s="48"/>
+      <c r="B33" s="61"/>
     </row>
     <row r="34" spans="1:3" ht="19.95" customHeight="1">
       <c r="A34" s="20" t="s">

</xml_diff>